<commit_message>
Improve MS-6 XLSX readability with Results sheet and clearer export semantics.
Add a compact Results worksheet, null unavailable error counts instead of zero, document 0-based frame indices with 1-based display columns, and regenerate committed outputs.
</commit_message>
<xml_diff>
--- a/outputs/test50_report.xlsx
+++ b/outputs/test50_report.xlsx
@@ -3,12 +3,21 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Summary" sheetId="1" r:id="rId1"/>
-    <sheet name="Events" sheetId="2" r:id="rId2"/>
-    <sheet name="Parameters" sheetId="3" r:id="rId3"/>
-    <sheet name="OperationalDefinitions" sheetId="4" r:id="rId4"/>
-    <sheet name="Provenance" sheetId="5" r:id="rId5"/>
+    <sheet name="Results" sheetId="1" r:id="rId1"/>
+    <sheet name="Summary" sheetId="2" r:id="rId2"/>
+    <sheet name="Events" sheetId="3" r:id="rId3"/>
+    <sheet name="Parameters" sheetId="4" r:id="rId4"/>
+    <sheet name="OperationalDefinitions" sheetId="5" r:id="rId5"/>
+    <sheet name="Provenance" sheetId="6" r:id="rId6"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Results'!A1:Z2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Summary'!A1:EV2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2">'Events'!A1:X62</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3">'Parameters'!A1:C42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4">'OperationalDefinitions'!A1:F17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5">'Provenance'!A1:U2</definedName>
+  </definedNames>
 </workbook>
 </file>
 
@@ -401,7 +410,361 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:Z2"/>
+  <cols>
+    <col min="1" max="1" width="18.83203125" customWidth="1"/>
+    <col min="2" max="2" width="12.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="10.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="28.83203125" customWidth="1"/>
+    <col min="8" max="8" width="44.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="16.83203125" customWidth="1"/>
+    <col min="11" max="11" width="16.83203125" customWidth="1"/>
+    <col min="12" max="12" width="16.83203125" customWidth="1"/>
+    <col min="13" max="13" width="16.83203125" customWidth="1"/>
+    <col min="14" max="14" width="14.83203125" customWidth="1"/>
+    <col min="15" max="15" width="14.83203125" customWidth="1"/>
+    <col min="16" max="16" width="14.83203125" customWidth="1"/>
+    <col min="17" max="17" width="14.83203125" customWidth="1"/>
+    <col min="18" max="18" width="14.83203125" customWidth="1"/>
+    <col min="19" max="19" width="12.83203125" customWidth="1"/>
+    <col min="20" max="20" width="12.83203125" customWidth="1"/>
+    <col min="21" max="21" width="18.83203125" customWidth="1"/>
+    <col min="22" max="22" width="18.83203125" customWidth="1"/>
+    <col min="23" max="23" width="18.83203125" customWidth="1"/>
+    <col min="24" max="24" width="18.83203125" customWidth="1"/>
+    <col min="25" max="25" width="14.83203125" customWidth="1"/>
+    <col min="26" max="26" width="16.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>fileName</v>
+      </c>
+      <c r="B1" t="str">
+        <v>label</v>
+      </c>
+      <c r="C1" t="str">
+        <v>measurementBasis</v>
+      </c>
+      <c r="D1" t="str">
+        <v>targetStatus</v>
+      </c>
+      <c r="E1" t="str">
+        <v>targetHole</v>
+      </c>
+      <c r="F1" t="str">
+        <v>scaleStatus</v>
+      </c>
+      <c r="G1" t="str">
+        <v>physicalScale</v>
+      </c>
+      <c r="H1" t="str">
+        <v>escapeState</v>
+      </c>
+      <c r="I1" t="str">
+        <v>eventsReviewStatus</v>
+      </c>
+      <c r="J1" t="str">
+        <v>primaryLatency</v>
+      </c>
+      <c r="K1" t="str">
+        <v>totalLatency</v>
+      </c>
+      <c r="L1" t="str">
+        <v>primaryErrors</v>
+      </c>
+      <c r="M1" t="str">
+        <v>totalErrors</v>
+      </c>
+      <c r="N1" t="str">
+        <v>primaryErrorsConfirmedCount</v>
+      </c>
+      <c r="O1" t="str">
+        <v>primaryErrorsProvisionalCount</v>
+      </c>
+      <c r="P1" t="str">
+        <v>totalErrorsConfirmedCount</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>totalErrorsProvisionalCount</v>
+      </c>
+      <c r="R1" t="str">
+        <v>pathLength</v>
+      </c>
+      <c r="S1" t="str">
+        <v>meanSpeed</v>
+      </c>
+      <c r="T1" t="str">
+        <v>maxSpeed</v>
+      </c>
+      <c r="U1" t="str">
+        <v>meanSpeedDiagnostic</v>
+      </c>
+      <c r="V1" t="str">
+        <v>maxSpeedDiagnostic</v>
+      </c>
+      <c r="W1" t="str">
+        <v>targetQuadrantFraction</v>
+      </c>
+      <c r="X1" t="str">
+        <v>targetQuadrantTime</v>
+      </c>
+      <c r="Y1" t="str">
+        <v>searchStrategy</v>
+      </c>
+      <c r="Z1" t="str">
+        <v>searchStrategyOverride</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>test50.mp4</v>
+      </c>
+      <c r="B2" t="str">
+        <v>test50</v>
+      </c>
+      <c r="C2" t="str">
+        <v>corrected</v>
+      </c>
+      <c r="D2" t="str">
+        <v>unknown</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Unknown</v>
+      </c>
+      <c r="F2" t="str">
+        <v>unknown</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Unknown (coordinates in px)</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Censored outcome — follow-up lower bound ≥ 180.033333 s</v>
+      </c>
+      <c r="I2" t="str">
+        <v>Current</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Unavailable (Target hole not confirmed.)</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Censored ≥ 180.03 s [escape_incomplete_censored]</v>
+      </c>
+      <c r="L2" t="str">
+        <v>Unavailable (Target hole not confirmed.)</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Unavailable (Target hole not confirmed.)</v>
+      </c>
+      <c r="N2" t="str">
+        <v>Target hole not confirmed.</v>
+      </c>
+      <c r="O2" t="str">
+        <v>Target hole not confirmed.</v>
+      </c>
+      <c r="P2" t="str">
+        <v>Target hole not confirmed.</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>Target hole not confirmed.</v>
+      </c>
+      <c r="R2" t="str">
+        <v>5909.99 px</v>
+      </c>
+      <c r="S2" t="str">
+        <v>31.66 px/s</v>
+      </c>
+      <c r="T2" t="str">
+        <v>226.95 px/s</v>
+      </c>
+      <c r="U2" t="str">
+        <v>31.89 px/s</v>
+      </c>
+      <c r="V2" t="str">
+        <v>79030.30 px/s</v>
+      </c>
+      <c r="W2" t="str">
+        <v>Unavailable (Target hole not confirmed.)</v>
+      </c>
+      <c r="X2" t="str">
+        <v>Unavailable (Target hole not confirmed.)</v>
+      </c>
+      <c r="Y2" t="str">
+        <v>random</v>
+      </c>
+      <c r="Z2" t="str">
+        <v>—</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:Z2"/>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z2"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:EV2"/>
+  <cols>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="14.83203125" customWidth="1"/>
+    <col min="8" max="8" width="14.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="10" max="10" width="14.83203125" customWidth="1"/>
+    <col min="11" max="11" width="14.83203125" customWidth="1"/>
+    <col min="12" max="12" width="14.83203125" customWidth="1"/>
+    <col min="13" max="13" width="14.83203125" customWidth="1"/>
+    <col min="14" max="14" width="14.83203125" customWidth="1"/>
+    <col min="15" max="15" width="14.83203125" customWidth="1"/>
+    <col min="16" max="16" width="14.83203125" customWidth="1"/>
+    <col min="17" max="17" width="14.83203125" customWidth="1"/>
+    <col min="18" max="18" width="14.83203125" customWidth="1"/>
+    <col min="19" max="19" width="14.83203125" customWidth="1"/>
+    <col min="20" max="20" width="14.83203125" customWidth="1"/>
+    <col min="21" max="21" width="14.83203125" customWidth="1"/>
+    <col min="22" max="22" width="14.83203125" customWidth="1"/>
+    <col min="23" max="23" width="14.83203125" customWidth="1"/>
+    <col min="24" max="24" width="14.83203125" customWidth="1"/>
+    <col min="25" max="25" width="14.83203125" customWidth="1"/>
+    <col min="26" max="26" width="14.83203125" customWidth="1"/>
+    <col min="27" max="27" width="14.83203125" customWidth="1"/>
+    <col min="28" max="28" width="14.83203125" customWidth="1"/>
+    <col min="29" max="29" width="14.83203125" customWidth="1"/>
+    <col min="30" max="30" width="14.83203125" customWidth="1"/>
+    <col min="31" max="31" width="14.83203125" customWidth="1"/>
+    <col min="32" max="32" width="14.83203125" customWidth="1"/>
+    <col min="33" max="33" width="14.83203125" customWidth="1"/>
+    <col min="34" max="34" width="14.83203125" customWidth="1"/>
+    <col min="35" max="35" width="14.83203125" customWidth="1"/>
+    <col min="36" max="36" width="14.83203125" customWidth="1"/>
+    <col min="37" max="37" width="14.83203125" customWidth="1"/>
+    <col min="38" max="38" width="14.83203125" customWidth="1"/>
+    <col min="39" max="39" width="14.83203125" customWidth="1"/>
+    <col min="40" max="40" width="14.83203125" customWidth="1"/>
+    <col min="41" max="41" width="14.83203125" customWidth="1"/>
+    <col min="42" max="42" width="14.83203125" customWidth="1"/>
+    <col min="43" max="43" width="14.83203125" customWidth="1"/>
+    <col min="44" max="44" width="14.83203125" customWidth="1"/>
+    <col min="45" max="45" width="14.83203125" customWidth="1"/>
+    <col min="46" max="46" width="14.83203125" customWidth="1"/>
+    <col min="47" max="47" width="14.83203125" customWidth="1"/>
+    <col min="48" max="48" width="14.83203125" customWidth="1"/>
+    <col min="49" max="49" width="14.83203125" customWidth="1"/>
+    <col min="50" max="50" width="14.83203125" customWidth="1"/>
+    <col min="51" max="51" width="14.83203125" customWidth="1"/>
+    <col min="52" max="52" width="14.83203125" customWidth="1"/>
+    <col min="53" max="53" width="14.83203125" customWidth="1"/>
+    <col min="54" max="54" width="14.83203125" customWidth="1"/>
+    <col min="55" max="55" width="14.83203125" customWidth="1"/>
+    <col min="56" max="56" width="14.83203125" customWidth="1"/>
+    <col min="57" max="57" width="14.83203125" customWidth="1"/>
+    <col min="58" max="58" width="14.83203125" customWidth="1"/>
+    <col min="59" max="59" width="14.83203125" customWidth="1"/>
+    <col min="60" max="60" width="14.83203125" customWidth="1"/>
+    <col min="61" max="61" width="14.83203125" customWidth="1"/>
+    <col min="62" max="62" width="14.83203125" customWidth="1"/>
+    <col min="63" max="63" width="14.83203125" customWidth="1"/>
+    <col min="64" max="64" width="14.83203125" customWidth="1"/>
+    <col min="65" max="65" width="14.83203125" customWidth="1"/>
+    <col min="66" max="66" width="14.83203125" customWidth="1"/>
+    <col min="67" max="67" width="14.83203125" customWidth="1"/>
+    <col min="68" max="68" width="14.83203125" customWidth="1"/>
+    <col min="69" max="69" width="14.83203125" customWidth="1"/>
+    <col min="70" max="70" width="14.83203125" customWidth="1"/>
+    <col min="71" max="71" width="14.83203125" customWidth="1"/>
+    <col min="72" max="72" width="14.83203125" customWidth="1"/>
+    <col min="73" max="73" width="14.83203125" customWidth="1"/>
+    <col min="74" max="74" width="14.83203125" customWidth="1"/>
+    <col min="75" max="75" width="14.83203125" customWidth="1"/>
+    <col min="76" max="76" width="14.83203125" customWidth="1"/>
+    <col min="77" max="77" width="14.83203125" customWidth="1"/>
+    <col min="78" max="78" width="14.83203125" customWidth="1"/>
+    <col min="79" max="79" width="14.83203125" customWidth="1"/>
+    <col min="80" max="80" width="14.83203125" customWidth="1"/>
+    <col min="81" max="81" width="14.83203125" customWidth="1"/>
+    <col min="82" max="82" width="14.83203125" customWidth="1"/>
+    <col min="83" max="83" width="14.83203125" customWidth="1"/>
+    <col min="84" max="84" width="14.83203125" customWidth="1"/>
+    <col min="85" max="85" width="14.83203125" customWidth="1"/>
+    <col min="86" max="86" width="14.83203125" customWidth="1"/>
+    <col min="87" max="87" width="14.83203125" customWidth="1"/>
+    <col min="88" max="88" width="14.83203125" customWidth="1"/>
+    <col min="89" max="89" width="14.83203125" customWidth="1"/>
+    <col min="90" max="90" width="14.83203125" customWidth="1"/>
+    <col min="91" max="91" width="14.83203125" customWidth="1"/>
+    <col min="92" max="92" width="14.83203125" customWidth="1"/>
+    <col min="93" max="93" width="14.83203125" customWidth="1"/>
+    <col min="94" max="94" width="14.83203125" customWidth="1"/>
+    <col min="95" max="95" width="14.83203125" customWidth="1"/>
+    <col min="96" max="96" width="14.83203125" customWidth="1"/>
+    <col min="97" max="97" width="14.83203125" customWidth="1"/>
+    <col min="98" max="98" width="14.83203125" customWidth="1"/>
+    <col min="99" max="99" width="14.83203125" customWidth="1"/>
+    <col min="100" max="100" width="14.83203125" customWidth="1"/>
+    <col min="101" max="101" width="14.83203125" customWidth="1"/>
+    <col min="102" max="102" width="14.83203125" customWidth="1"/>
+    <col min="103" max="103" width="14.83203125" customWidth="1"/>
+    <col min="104" max="104" width="14.83203125" customWidth="1"/>
+    <col min="105" max="105" width="14.83203125" customWidth="1"/>
+    <col min="106" max="106" width="14.83203125" customWidth="1"/>
+    <col min="107" max="107" width="14.83203125" customWidth="1"/>
+    <col min="108" max="108" width="14.83203125" customWidth="1"/>
+    <col min="109" max="109" width="14.83203125" customWidth="1"/>
+    <col min="110" max="110" width="14.83203125" customWidth="1"/>
+    <col min="111" max="111" width="14.83203125" customWidth="1"/>
+    <col min="112" max="112" width="14.83203125" customWidth="1"/>
+    <col min="113" max="113" width="14.83203125" customWidth="1"/>
+    <col min="114" max="114" width="14.83203125" customWidth="1"/>
+    <col min="115" max="115" width="14.83203125" customWidth="1"/>
+    <col min="116" max="116" width="14.83203125" customWidth="1"/>
+    <col min="117" max="117" width="14.83203125" customWidth="1"/>
+    <col min="118" max="118" width="14.83203125" customWidth="1"/>
+    <col min="119" max="119" width="14.83203125" customWidth="1"/>
+    <col min="120" max="120" width="14.83203125" customWidth="1"/>
+    <col min="121" max="121" width="14.83203125" customWidth="1"/>
+    <col min="122" max="122" width="14.83203125" customWidth="1"/>
+    <col min="123" max="123" width="14.83203125" customWidth="1"/>
+    <col min="124" max="124" width="14.83203125" customWidth="1"/>
+    <col min="125" max="125" width="14.83203125" customWidth="1"/>
+    <col min="126" max="126" width="14.83203125" customWidth="1"/>
+    <col min="127" max="127" width="14.83203125" customWidth="1"/>
+    <col min="128" max="128" width="14.83203125" customWidth="1"/>
+    <col min="129" max="129" width="14.83203125" customWidth="1"/>
+    <col min="130" max="130" width="14.83203125" customWidth="1"/>
+    <col min="131" max="131" width="14.83203125" customWidth="1"/>
+    <col min="132" max="132" width="14.83203125" customWidth="1"/>
+    <col min="133" max="133" width="14.83203125" customWidth="1"/>
+    <col min="134" max="134" width="14.83203125" customWidth="1"/>
+    <col min="135" max="135" width="14.83203125" customWidth="1"/>
+    <col min="136" max="136" width="14.83203125" customWidth="1"/>
+    <col min="137" max="137" width="14.83203125" customWidth="1"/>
+    <col min="138" max="138" width="14.83203125" customWidth="1"/>
+    <col min="139" max="139" width="14.83203125" customWidth="1"/>
+    <col min="140" max="140" width="14.83203125" customWidth="1"/>
+    <col min="141" max="141" width="14.83203125" customWidth="1"/>
+    <col min="142" max="142" width="14.83203125" customWidth="1"/>
+    <col min="143" max="143" width="14.83203125" customWidth="1"/>
+    <col min="144" max="144" width="14.83203125" customWidth="1"/>
+    <col min="145" max="145" width="14.83203125" customWidth="1"/>
+    <col min="146" max="146" width="14.83203125" customWidth="1"/>
+    <col min="147" max="147" width="14.83203125" customWidth="1"/>
+    <col min="148" max="148" width="14.83203125" customWidth="1"/>
+    <col min="149" max="149" width="14.83203125" customWidth="1"/>
+    <col min="150" max="150" width="14.83203125" customWidth="1"/>
+    <col min="151" max="151" width="14.83203125" customWidth="1"/>
+    <col min="152" max="152" width="14.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -896,7 +1259,7 @@
         <v>2026-09-07T18:13:26.622Z</v>
       </c>
       <c r="P2" t="str">
-        <v>2026-09-07T19:54:09.012Z</v>
+        <v>2026-09-07T20:08:18.628Z</v>
       </c>
       <c r="Q2" t="str">
         <v>false</v>
@@ -907,18 +1270,6 @@
       <c r="T2" t="str">
         <v>random</v>
       </c>
-      <c r="V2">
-        <v>0</v>
-      </c>
-      <c r="W2">
-        <v>0</v>
-      </c>
-      <c r="X2">
-        <v>0</v>
-      </c>
-      <c r="Y2">
-        <v>0</v>
-      </c>
       <c r="AA2" t="str">
         <v>unavailable</v>
       </c>
@@ -1164,129 +1515,118 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:EV2"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:EV2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:V61"/>
+  <dimension ref="A1:X62"/>
+  <cols>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="36.83203125" customWidth="1"/>
+    <col min="3" max="3" width="22.83203125" customWidth="1"/>
+    <col min="4" max="4" width="28.83203125" customWidth="1"/>
+    <col min="5" max="5" width="10.83203125" customWidth="1"/>
+    <col min="6" max="6" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="18.83203125" customWidth="1"/>
+    <col min="8" max="8" width="18.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="16.83203125" customWidth="1"/>
+    <col min="12" max="12" width="16.83203125" customWidth="1"/>
+    <col min="13" max="13" width="16.83203125" customWidth="1"/>
+    <col min="14" max="14" width="10.83203125" customWidth="1"/>
+    <col min="15" max="15" width="12.83203125" customWidth="1"/>
+    <col min="16" max="16" width="12.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="10.83203125" customWidth="1"/>
+    <col min="19" max="19" width="14.83203125" customWidth="1"/>
+    <col min="20" max="20" width="14.83203125" customWidth="1"/>
+    <col min="21" max="21" width="18.83203125" customWidth="1"/>
+    <col min="22" max="22" width="24.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>trialId</v>
-      </c>
-      <c r="B1" t="str">
-        <v>eventId</v>
-      </c>
-      <c r="C1" t="str">
-        <v>type</v>
-      </c>
-      <c r="D1" t="str">
-        <v>exportLabel</v>
-      </c>
-      <c r="E1" t="str">
-        <v>holeDisplay</v>
-      </c>
-      <c r="F1" t="str">
-        <v>holeIdInternal</v>
-      </c>
-      <c r="G1" t="str">
-        <v>startFrameIndex</v>
-      </c>
-      <c r="H1" t="str">
-        <v>endFrameIndex</v>
-      </c>
-      <c r="I1" t="str">
-        <v>startTimeSec</v>
-      </c>
-      <c r="J1" t="str">
-        <v>endTimeSec</v>
-      </c>
-      <c r="K1" t="str">
-        <v>entryOnsetTimeSec</v>
-      </c>
-      <c r="L1" t="str">
-        <v>completionTimeSec</v>
-      </c>
-      <c r="M1" t="str">
-        <v>censorBoundaryTimeSec</v>
-      </c>
-      <c r="N1" t="str">
-        <v>origin</v>
-      </c>
-      <c r="O1" t="str">
-        <v>status</v>
-      </c>
-      <c r="P1" t="str">
-        <v>confidence</v>
-      </c>
-      <c r="Q1" t="str">
-        <v>visitIndex</v>
-      </c>
-      <c r="R1" t="str">
-        <v>isRevisit</v>
-      </c>
-      <c r="S1" t="str">
-        <v>bodyEntryPath</v>
-      </c>
-      <c r="T1" t="str">
-        <v>bodyEntryVersion</v>
-      </c>
-      <c r="U1" t="str">
-        <v>pixelEvidenceComplete</v>
-      </c>
-      <c r="V1" t="str">
-        <v>notes</v>
+        <v>Frame indices: startFrameIndex and endFrameIndex are 0-based internal decoder indices. startFrameDisplay and endFrameDisplay add 1 for human-readable frame numbers.</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
+        <v>trialId</v>
       </c>
       <c r="B2" t="str">
-        <v>c0b3f98e-fbec-47a9-aba5-8a6c9b24716e</v>
+        <v>eventId</v>
       </c>
       <c r="C2" t="str">
-        <v>investigation</v>
+        <v>type</v>
       </c>
       <c r="D2" t="str">
-        <v>investigation</v>
-      </c>
-      <c r="E2">
-        <v>5</v>
-      </c>
-      <c r="F2">
-        <v>4</v>
-      </c>
-      <c r="G2">
-        <v>188</v>
-      </c>
-      <c r="H2">
-        <v>301</v>
-      </c>
-      <c r="I2">
-        <v>6.333333</v>
-      </c>
-      <c r="J2">
-        <v>10.133333</v>
+        <v>exportLabel</v>
+      </c>
+      <c r="E2" t="str">
+        <v>holeDisplay</v>
+      </c>
+      <c r="F2" t="str">
+        <v>holeIdInternal</v>
+      </c>
+      <c r="G2" t="str">
+        <v>startFrameIndex</v>
+      </c>
+      <c r="H2" t="str">
+        <v>endFrameIndex</v>
+      </c>
+      <c r="I2" t="str">
+        <v>startFrameDisplay</v>
+      </c>
+      <c r="J2" t="str">
+        <v>endFrameDisplay</v>
+      </c>
+      <c r="K2" t="str">
+        <v>startTimeSec</v>
+      </c>
+      <c r="L2" t="str">
+        <v>endTimeSec</v>
+      </c>
+      <c r="M2" t="str">
+        <v>entryOnsetTimeSec</v>
       </c>
       <c r="N2" t="str">
-        <v>auto</v>
+        <v>completionTimeSec</v>
       </c>
       <c r="O2" t="str">
-        <v>proposed</v>
+        <v>censorBoundaryTimeSec</v>
       </c>
       <c r="P2" t="str">
-        <v>medium</v>
-      </c>
-      <c r="Q2">
-        <v>1</v>
+        <v>origin</v>
+      </c>
+      <c r="Q2" t="str">
+        <v>status</v>
       </c>
       <c r="R2" t="str">
-        <v>false</v>
+        <v>confidence</v>
+      </c>
+      <c r="S2" t="str">
+        <v>visitIndex</v>
+      </c>
+      <c r="T2" t="str">
+        <v>isRevisit</v>
+      </c>
+      <c r="U2" t="str">
+        <v>bodyEntryPath</v>
+      </c>
+      <c r="V2" t="str">
+        <v>bodyEntryVersion</v>
+      </c>
+      <c r="W2" t="str">
+        <v>pixelEvidenceComplete</v>
+      </c>
+      <c r="X2" t="str">
+        <v>notes</v>
       </c>
     </row>
     <row r="3">
@@ -1294,7 +1634,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B3" t="str">
-        <v>d602e2ca-5d8a-498b-bb97-92045cf2a129</v>
+        <v>c0b3f98e-fbec-47a9-aba5-8a6c9b24716e</v>
       </c>
       <c r="C3" t="str">
         <v>investigation</v>
@@ -1303,36 +1643,42 @@
         <v>investigation</v>
       </c>
       <c r="E3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G3">
-        <v>309</v>
+        <v>188</v>
       </c>
       <c r="H3">
-        <v>395</v>
+        <v>301</v>
       </c>
       <c r="I3">
-        <v>10.4</v>
+        <v>189</v>
       </c>
       <c r="J3">
-        <v>13.266667</v>
-      </c>
-      <c r="N3" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O3" t="str">
-        <v>proposed</v>
+        <v>302</v>
+      </c>
+      <c r="K3">
+        <v>6.333333</v>
+      </c>
+      <c r="L3">
+        <v>10.133333</v>
       </c>
       <c r="P3" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R3" t="str">
         <v>medium</v>
       </c>
-      <c r="Q3">
+      <c r="S3">
         <v>1</v>
       </c>
-      <c r="R3" t="str">
+      <c r="T3" t="str">
         <v>false</v>
       </c>
     </row>
@@ -1341,7 +1687,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B4" t="str">
-        <v>4cb42db9-2937-44f8-b94b-893bdde43b8c</v>
+        <v>d602e2ca-5d8a-498b-bb97-92045cf2a129</v>
       </c>
       <c r="C4" t="str">
         <v>investigation</v>
@@ -1356,31 +1702,37 @@
         <v>5</v>
       </c>
       <c r="G4">
-        <v>434</v>
+        <v>309</v>
       </c>
       <c r="H4">
-        <v>472</v>
+        <v>395</v>
       </c>
       <c r="I4">
-        <v>14.566667</v>
+        <v>310</v>
       </c>
       <c r="J4">
-        <v>15.833333</v>
-      </c>
-      <c r="N4" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O4" t="str">
-        <v>proposed</v>
+        <v>396</v>
+      </c>
+      <c r="K4">
+        <v>10.4</v>
+      </c>
+      <c r="L4">
+        <v>13.266667</v>
       </c>
       <c r="P4" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R4" t="str">
         <v>medium</v>
       </c>
-      <c r="Q4">
-        <v>2</v>
-      </c>
-      <c r="R4" t="str">
-        <v>true</v>
+      <c r="S4">
+        <v>1</v>
+      </c>
+      <c r="T4" t="str">
+        <v>false</v>
       </c>
     </row>
     <row r="5">
@@ -1388,7 +1740,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B5" t="str">
-        <v>863579b8-c4db-4b30-90c7-219838218030</v>
+        <v>4cb42db9-2937-44f8-b94b-893bdde43b8c</v>
       </c>
       <c r="C5" t="str">
         <v>investigation</v>
@@ -1397,37 +1749,43 @@
         <v>investigation</v>
       </c>
       <c r="E5">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F5">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G5">
-        <v>475</v>
+        <v>434</v>
       </c>
       <c r="H5">
-        <v>548</v>
+        <v>472</v>
       </c>
       <c r="I5">
-        <v>15.933333</v>
+        <v>435</v>
       </c>
       <c r="J5">
-        <v>18.366667</v>
-      </c>
-      <c r="N5" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O5" t="str">
-        <v>proposed</v>
+        <v>473</v>
+      </c>
+      <c r="K5">
+        <v>14.566667</v>
+      </c>
+      <c r="L5">
+        <v>15.833333</v>
       </c>
       <c r="P5" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q5" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R5" t="str">
         <v>medium</v>
       </c>
-      <c r="Q5">
-        <v>1</v>
-      </c>
-      <c r="R5" t="str">
-        <v>false</v>
+      <c r="S5">
+        <v>2</v>
+      </c>
+      <c r="T5" t="str">
+        <v>true</v>
       </c>
     </row>
     <row r="6">
@@ -1435,7 +1793,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B6" t="str">
-        <v>ebf87c26-be89-47eb-a25e-2eabd47a385a</v>
+        <v>863579b8-c4db-4b30-90c7-219838218030</v>
       </c>
       <c r="C6" t="str">
         <v>investigation</v>
@@ -1450,31 +1808,37 @@
         <v>6</v>
       </c>
       <c r="G6">
-        <v>558</v>
+        <v>475</v>
       </c>
       <c r="H6">
-        <v>571</v>
+        <v>548</v>
       </c>
       <c r="I6">
-        <v>18.700065</v>
+        <v>476</v>
       </c>
       <c r="J6">
-        <v>19.133333</v>
-      </c>
-      <c r="N6" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O6" t="str">
-        <v>proposed</v>
+        <v>549</v>
+      </c>
+      <c r="K6">
+        <v>15.933333</v>
+      </c>
+      <c r="L6">
+        <v>18.366667</v>
       </c>
       <c r="P6" t="str">
-        <v>low</v>
-      </c>
-      <c r="Q6">
-        <v>2</v>
+        <v>auto</v>
+      </c>
+      <c r="Q6" t="str">
+        <v>proposed</v>
       </c>
       <c r="R6" t="str">
-        <v>true</v>
+        <v>medium</v>
+      </c>
+      <c r="S6">
+        <v>1</v>
+      </c>
+      <c r="T6" t="str">
+        <v>false</v>
       </c>
     </row>
     <row r="7">
@@ -1482,7 +1846,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B7" t="str">
-        <v>e3c02d4c-5690-4403-a381-ef8c1357360c</v>
+        <v>ebf87c26-be89-47eb-a25e-2eabd47a385a</v>
       </c>
       <c r="C7" t="str">
         <v>investigation</v>
@@ -1497,30 +1861,36 @@
         <v>6</v>
       </c>
       <c r="G7">
-        <v>592</v>
+        <v>558</v>
       </c>
       <c r="H7">
-        <v>698</v>
+        <v>571</v>
       </c>
       <c r="I7">
-        <v>19.866667</v>
+        <v>559</v>
       </c>
       <c r="J7">
-        <v>23.4</v>
-      </c>
-      <c r="N7" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O7" t="str">
-        <v>proposed</v>
+        <v>572</v>
+      </c>
+      <c r="K7">
+        <v>18.700065</v>
+      </c>
+      <c r="L7">
+        <v>19.133333</v>
       </c>
       <c r="P7" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q7" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R7" t="str">
         <v>low</v>
       </c>
-      <c r="Q7">
-        <v>3</v>
-      </c>
-      <c r="R7" t="str">
+      <c r="S7">
+        <v>2</v>
+      </c>
+      <c r="T7" t="str">
         <v>true</v>
       </c>
     </row>
@@ -1529,7 +1899,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B8" t="str">
-        <v>ba4b1aca-34ae-49f5-a98a-3f8e281948b3</v>
+        <v>e3c02d4c-5690-4403-a381-ef8c1357360c</v>
       </c>
       <c r="C8" t="str">
         <v>investigation</v>
@@ -1538,37 +1908,43 @@
         <v>investigation</v>
       </c>
       <c r="E8">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F8">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G8">
+        <v>592</v>
+      </c>
+      <c r="H8">
+        <v>698</v>
+      </c>
+      <c r="I8">
+        <v>593</v>
+      </c>
+      <c r="J8">
         <v>699</v>
       </c>
-      <c r="H8">
-        <v>867</v>
-      </c>
-      <c r="I8">
-        <v>23.433333</v>
-      </c>
-      <c r="J8">
-        <v>29.033333</v>
-      </c>
-      <c r="N8" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O8" t="str">
-        <v>proposed</v>
+      <c r="K8">
+        <v>19.866667</v>
+      </c>
+      <c r="L8">
+        <v>23.4</v>
       </c>
       <c r="P8" t="str">
-        <v>medium</v>
-      </c>
-      <c r="Q8">
-        <v>1</v>
+        <v>auto</v>
+      </c>
+      <c r="Q8" t="str">
+        <v>proposed</v>
       </c>
       <c r="R8" t="str">
-        <v>false</v>
+        <v>low</v>
+      </c>
+      <c r="S8">
+        <v>3</v>
+      </c>
+      <c r="T8" t="str">
+        <v>true</v>
       </c>
     </row>
     <row r="9">
@@ -1576,7 +1952,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B9" t="str">
-        <v>060521ec-af3b-40dc-9122-2e81f1fb0829</v>
+        <v>ba4b1aca-34ae-49f5-a98a-3f8e281948b3</v>
       </c>
       <c r="C9" t="str">
         <v>investigation</v>
@@ -1585,36 +1961,42 @@
         <v>investigation</v>
       </c>
       <c r="E9">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F9">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G9">
+        <v>699</v>
+      </c>
+      <c r="H9">
+        <v>867</v>
+      </c>
+      <c r="I9">
+        <v>700</v>
+      </c>
+      <c r="J9">
         <v>868</v>
       </c>
-      <c r="H9">
-        <v>905</v>
-      </c>
-      <c r="I9">
-        <v>29.066667</v>
-      </c>
-      <c r="J9">
-        <v>30.3</v>
-      </c>
-      <c r="N9" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O9" t="str">
-        <v>proposed</v>
+      <c r="K9">
+        <v>23.433333</v>
+      </c>
+      <c r="L9">
+        <v>29.033333</v>
       </c>
       <c r="P9" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q9" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R9" t="str">
         <v>medium</v>
       </c>
-      <c r="Q9">
+      <c r="S9">
         <v>1</v>
       </c>
-      <c r="R9" t="str">
+      <c r="T9" t="str">
         <v>false</v>
       </c>
     </row>
@@ -1623,7 +2005,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B10" t="str">
-        <v>55663664-de20-4023-a39a-449591f9c50b</v>
+        <v>060521ec-af3b-40dc-9122-2e81f1fb0829</v>
       </c>
       <c r="C10" t="str">
         <v>investigation</v>
@@ -1632,36 +2014,42 @@
         <v>investigation</v>
       </c>
       <c r="E10">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F10">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G10">
-        <v>913</v>
+        <v>868</v>
       </c>
       <c r="H10">
-        <v>943</v>
+        <v>905</v>
       </c>
       <c r="I10">
-        <v>30.566667</v>
+        <v>869</v>
       </c>
       <c r="J10">
-        <v>31.566667</v>
-      </c>
-      <c r="N10" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O10" t="str">
-        <v>proposed</v>
+        <v>906</v>
+      </c>
+      <c r="K10">
+        <v>29.066667</v>
+      </c>
+      <c r="L10">
+        <v>30.3</v>
       </c>
       <c r="P10" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q10" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R10" t="str">
         <v>medium</v>
       </c>
-      <c r="Q10">
+      <c r="S10">
         <v>1</v>
       </c>
-      <c r="R10" t="str">
+      <c r="T10" t="str">
         <v>false</v>
       </c>
     </row>
@@ -1670,7 +2058,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B11" t="str">
-        <v>2f55c07b-d87c-487f-b846-582ab0049b28</v>
+        <v>55663664-de20-4023-a39a-449591f9c50b</v>
       </c>
       <c r="C11" t="str">
         <v>investigation</v>
@@ -1685,31 +2073,37 @@
         <v>9</v>
       </c>
       <c r="G11">
-        <v>947</v>
+        <v>913</v>
       </c>
       <c r="H11">
-        <v>986</v>
+        <v>943</v>
       </c>
       <c r="I11">
-        <v>31.7</v>
+        <v>914</v>
       </c>
       <c r="J11">
-        <v>33</v>
-      </c>
-      <c r="N11" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O11" t="str">
-        <v>proposed</v>
+        <v>944</v>
+      </c>
+      <c r="K11">
+        <v>30.566667</v>
+      </c>
+      <c r="L11">
+        <v>31.566667</v>
       </c>
       <c r="P11" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q11" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R11" t="str">
         <v>medium</v>
       </c>
-      <c r="Q11">
-        <v>2</v>
-      </c>
-      <c r="R11" t="str">
-        <v>true</v>
+      <c r="S11">
+        <v>1</v>
+      </c>
+      <c r="T11" t="str">
+        <v>false</v>
       </c>
     </row>
     <row r="12">
@@ -1717,7 +2111,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B12" t="str">
-        <v>6ac94f42-46c8-4680-be1f-07d227165b61</v>
+        <v>2f55c07b-d87c-487f-b846-582ab0049b28</v>
       </c>
       <c r="C12" t="str">
         <v>investigation</v>
@@ -1726,37 +2120,43 @@
         <v>investigation</v>
       </c>
       <c r="E12">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F12">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G12">
-        <v>997</v>
+        <v>947</v>
       </c>
       <c r="H12">
-        <v>1025</v>
+        <v>986</v>
       </c>
       <c r="I12">
-        <v>33.366667</v>
+        <v>948</v>
       </c>
       <c r="J12">
-        <v>34.300065</v>
-      </c>
-      <c r="N12" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O12" t="str">
-        <v>proposed</v>
+        <v>987</v>
+      </c>
+      <c r="K12">
+        <v>31.7</v>
+      </c>
+      <c r="L12">
+        <v>33</v>
       </c>
       <c r="P12" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q12" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R12" t="str">
         <v>medium</v>
       </c>
-      <c r="Q12">
-        <v>1</v>
-      </c>
-      <c r="R12" t="str">
-        <v>false</v>
+      <c r="S12">
+        <v>2</v>
+      </c>
+      <c r="T12" t="str">
+        <v>true</v>
       </c>
     </row>
     <row r="13">
@@ -1764,7 +2164,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B13" t="str">
-        <v>833e5425-931d-4434-8fb3-c1519f757f60</v>
+        <v>6ac94f42-46c8-4680-be1f-07d227165b61</v>
       </c>
       <c r="C13" t="str">
         <v>investigation</v>
@@ -1773,36 +2173,42 @@
         <v>investigation</v>
       </c>
       <c r="E13">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F13">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G13">
-        <v>1049</v>
+        <v>997</v>
       </c>
       <c r="H13">
-        <v>1136</v>
+        <v>1025</v>
       </c>
       <c r="I13">
-        <v>35.1</v>
+        <v>998</v>
       </c>
       <c r="J13">
-        <v>38.033333</v>
-      </c>
-      <c r="N13" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O13" t="str">
-        <v>proposed</v>
+        <v>1026</v>
+      </c>
+      <c r="K13">
+        <v>33.366667</v>
+      </c>
+      <c r="L13">
+        <v>34.300065</v>
       </c>
       <c r="P13" t="str">
-        <v>low</v>
-      </c>
-      <c r="Q13">
+        <v>auto</v>
+      </c>
+      <c r="Q13" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R13" t="str">
+        <v>medium</v>
+      </c>
+      <c r="S13">
         <v>1</v>
       </c>
-      <c r="R13" t="str">
+      <c r="T13" t="str">
         <v>false</v>
       </c>
     </row>
@@ -1811,7 +2217,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B14" t="str">
-        <v>9de7f218-3174-4f54-b6f6-c51ee1963fe5</v>
+        <v>833e5425-931d-4434-8fb3-c1519f757f60</v>
       </c>
       <c r="C14" t="str">
         <v>investigation</v>
@@ -1820,37 +2226,43 @@
         <v>investigation</v>
       </c>
       <c r="E14">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="F14">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="G14">
-        <v>1341</v>
+        <v>1049</v>
       </c>
       <c r="H14">
-        <v>1469</v>
+        <v>1136</v>
       </c>
       <c r="I14">
-        <v>44.866667</v>
+        <v>1050</v>
       </c>
       <c r="J14">
-        <v>49.133333</v>
-      </c>
-      <c r="N14" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O14" t="str">
-        <v>proposed</v>
+        <v>1137</v>
+      </c>
+      <c r="K14">
+        <v>35.1</v>
+      </c>
+      <c r="L14">
+        <v>38.033333</v>
       </c>
       <c r="P14" t="str">
-        <v>medium</v>
-      </c>
-      <c r="Q14">
-        <v>3</v>
+        <v>auto</v>
+      </c>
+      <c r="Q14" t="str">
+        <v>proposed</v>
       </c>
       <c r="R14" t="str">
-        <v>true</v>
+        <v>low</v>
+      </c>
+      <c r="S14">
+        <v>1</v>
+      </c>
+      <c r="T14" t="str">
+        <v>false</v>
       </c>
     </row>
     <row r="15">
@@ -1858,7 +2270,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B15" t="str">
-        <v>e5e733ff-fdb1-4913-acb0-bb2343719e44</v>
+        <v>9de7f218-3174-4f54-b6f6-c51ee1963fe5</v>
       </c>
       <c r="C15" t="str">
         <v>investigation</v>
@@ -1867,36 +2279,42 @@
         <v>investigation</v>
       </c>
       <c r="E15">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F15">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G15">
+        <v>1341</v>
+      </c>
+      <c r="H15">
+        <v>1469</v>
+      </c>
+      <c r="I15">
+        <v>1342</v>
+      </c>
+      <c r="J15">
         <v>1470</v>
       </c>
-      <c r="H15">
-        <v>1551</v>
-      </c>
-      <c r="I15">
-        <v>49.166667</v>
-      </c>
-      <c r="J15">
-        <v>51.866667</v>
-      </c>
-      <c r="N15" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O15" t="str">
-        <v>proposed</v>
+      <c r="K15">
+        <v>44.866667</v>
+      </c>
+      <c r="L15">
+        <v>49.133333</v>
       </c>
       <c r="P15" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q15" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R15" t="str">
         <v>medium</v>
       </c>
-      <c r="Q15">
-        <v>4</v>
-      </c>
-      <c r="R15" t="str">
+      <c r="S15">
+        <v>3</v>
+      </c>
+      <c r="T15" t="str">
         <v>true</v>
       </c>
     </row>
@@ -1905,7 +2323,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B16" t="str">
-        <v>9c0176ab-be9a-4a89-8778-a18737a34125</v>
+        <v>e5e733ff-fdb1-4913-acb0-bb2343719e44</v>
       </c>
       <c r="C16" t="str">
         <v>investigation</v>
@@ -1914,36 +2332,42 @@
         <v>investigation</v>
       </c>
       <c r="E16">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F16">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G16">
-        <v>1555</v>
+        <v>1470</v>
       </c>
       <c r="H16">
-        <v>1602</v>
+        <v>1551</v>
       </c>
       <c r="I16">
-        <v>52.033333</v>
+        <v>1471</v>
       </c>
       <c r="J16">
-        <v>53.6</v>
-      </c>
-      <c r="N16" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O16" t="str">
-        <v>proposed</v>
+        <v>1552</v>
+      </c>
+      <c r="K16">
+        <v>49.166667</v>
+      </c>
+      <c r="L16">
+        <v>51.866667</v>
       </c>
       <c r="P16" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q16" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R16" t="str">
         <v>medium</v>
       </c>
-      <c r="Q16">
-        <v>2</v>
-      </c>
-      <c r="R16" t="str">
+      <c r="S16">
+        <v>4</v>
+      </c>
+      <c r="T16" t="str">
         <v>true</v>
       </c>
     </row>
@@ -1952,7 +2376,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B17" t="str">
-        <v>ee124390-b7cf-45d3-9cef-c90063b0583b</v>
+        <v>9c0176ab-be9a-4a89-8778-a18737a34125</v>
       </c>
       <c r="C17" t="str">
         <v>investigation</v>
@@ -1961,36 +2385,42 @@
         <v>investigation</v>
       </c>
       <c r="E17">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F17">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G17">
-        <v>1605</v>
+        <v>1555</v>
       </c>
       <c r="H17">
-        <v>1630</v>
+        <v>1602</v>
       </c>
       <c r="I17">
-        <v>53.7</v>
+        <v>1556</v>
       </c>
       <c r="J17">
-        <v>54.533333</v>
-      </c>
-      <c r="N17" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O17" t="str">
-        <v>proposed</v>
+        <v>1603</v>
+      </c>
+      <c r="K17">
+        <v>52.033333</v>
+      </c>
+      <c r="L17">
+        <v>53.6</v>
       </c>
       <c r="P17" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q17" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R17" t="str">
         <v>medium</v>
       </c>
-      <c r="Q17">
+      <c r="S17">
         <v>2</v>
       </c>
-      <c r="R17" t="str">
+      <c r="T17" t="str">
         <v>true</v>
       </c>
     </row>
@@ -1999,7 +2429,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B18" t="str">
-        <v>bff02d54-af3f-4560-8981-08697e45f648</v>
+        <v>ee124390-b7cf-45d3-9cef-c90063b0583b</v>
       </c>
       <c r="C18" t="str">
         <v>investigation</v>
@@ -2008,36 +2438,42 @@
         <v>investigation</v>
       </c>
       <c r="E18">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F18">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G18">
-        <v>1721</v>
+        <v>1605</v>
       </c>
       <c r="H18">
-        <v>1778</v>
+        <v>1630</v>
       </c>
       <c r="I18">
-        <v>57.566667</v>
+        <v>1606</v>
       </c>
       <c r="J18">
-        <v>59.466667</v>
-      </c>
-      <c r="N18" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O18" t="str">
-        <v>proposed</v>
+        <v>1631</v>
+      </c>
+      <c r="K18">
+        <v>53.7</v>
+      </c>
+      <c r="L18">
+        <v>54.533333</v>
       </c>
       <c r="P18" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q18" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R18" t="str">
         <v>medium</v>
       </c>
-      <c r="Q18">
-        <v>3</v>
-      </c>
-      <c r="R18" t="str">
+      <c r="S18">
+        <v>2</v>
+      </c>
+      <c r="T18" t="str">
         <v>true</v>
       </c>
     </row>
@@ -2046,7 +2482,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B19" t="str">
-        <v>04c30f57-7d7f-4727-b999-642f436c77b8</v>
+        <v>bff02d54-af3f-4560-8981-08697e45f648</v>
       </c>
       <c r="C19" t="str">
         <v>investigation</v>
@@ -2055,36 +2491,42 @@
         <v>investigation</v>
       </c>
       <c r="E19">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F19">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G19">
-        <v>1787</v>
+        <v>1721</v>
       </c>
       <c r="H19">
-        <v>1811</v>
+        <v>1778</v>
       </c>
       <c r="I19">
-        <v>59.766667</v>
+        <v>1722</v>
       </c>
       <c r="J19">
-        <v>60.566667</v>
-      </c>
-      <c r="N19" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O19" t="str">
-        <v>proposed</v>
+        <v>1779</v>
+      </c>
+      <c r="K19">
+        <v>57.566667</v>
+      </c>
+      <c r="L19">
+        <v>59.466667</v>
       </c>
       <c r="P19" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q19" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R19" t="str">
         <v>medium</v>
       </c>
-      <c r="Q19">
-        <v>2</v>
-      </c>
-      <c r="R19" t="str">
+      <c r="S19">
+        <v>3</v>
+      </c>
+      <c r="T19" t="str">
         <v>true</v>
       </c>
     </row>
@@ -2093,7 +2535,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B20" t="str">
-        <v>e9848d71-fa19-42ab-8b7c-8d5873355053</v>
+        <v>04c30f57-7d7f-4727-b999-642f436c77b8</v>
       </c>
       <c r="C20" t="str">
         <v>investigation</v>
@@ -2102,36 +2544,42 @@
         <v>investigation</v>
       </c>
       <c r="E20">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F20">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G20">
-        <v>1836</v>
+        <v>1787</v>
       </c>
       <c r="H20">
-        <v>1937</v>
+        <v>1811</v>
       </c>
       <c r="I20">
-        <v>61.4</v>
+        <v>1788</v>
       </c>
       <c r="J20">
-        <v>64.766667</v>
-      </c>
-      <c r="N20" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O20" t="str">
-        <v>proposed</v>
+        <v>1812</v>
+      </c>
+      <c r="K20">
+        <v>59.766667</v>
+      </c>
+      <c r="L20">
+        <v>60.566667</v>
       </c>
       <c r="P20" t="str">
-        <v>low</v>
-      </c>
-      <c r="Q20">
+        <v>auto</v>
+      </c>
+      <c r="Q20" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R20" t="str">
+        <v>medium</v>
+      </c>
+      <c r="S20">
         <v>2</v>
       </c>
-      <c r="R20" t="str">
+      <c r="T20" t="str">
         <v>true</v>
       </c>
     </row>
@@ -2140,7 +2588,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B21" t="str">
-        <v>6d537e54-9f0a-4433-b3dc-8b6230d3cec5</v>
+        <v>e9848d71-fa19-42ab-8b7c-8d5873355053</v>
       </c>
       <c r="C21" t="str">
         <v>investigation</v>
@@ -2149,37 +2597,43 @@
         <v>investigation</v>
       </c>
       <c r="E21">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F21">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G21">
-        <v>1960</v>
+        <v>1836</v>
       </c>
       <c r="H21">
-        <v>1986</v>
+        <v>1937</v>
       </c>
       <c r="I21">
-        <v>65.533333</v>
+        <v>1837</v>
       </c>
       <c r="J21">
-        <v>66.433333</v>
-      </c>
-      <c r="N21" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O21" t="str">
-        <v>proposed</v>
+        <v>1938</v>
+      </c>
+      <c r="K21">
+        <v>61.4</v>
+      </c>
+      <c r="L21">
+        <v>64.766667</v>
       </c>
       <c r="P21" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q21" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R21" t="str">
         <v>low</v>
       </c>
-      <c r="Q21">
-        <v>1</v>
-      </c>
-      <c r="R21" t="str">
-        <v>false</v>
+      <c r="S21">
+        <v>2</v>
+      </c>
+      <c r="T21" t="str">
+        <v>true</v>
       </c>
     </row>
     <row r="22">
@@ -2187,7 +2641,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B22" t="str">
-        <v>23dce394-981c-4a8e-9eb0-aa66349c9912</v>
+        <v>6d537e54-9f0a-4433-b3dc-8b6230d3cec5</v>
       </c>
       <c r="C22" t="str">
         <v>investigation</v>
@@ -2196,36 +2650,42 @@
         <v>investigation</v>
       </c>
       <c r="E22">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F22">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G22">
-        <v>2000</v>
+        <v>1960</v>
       </c>
       <c r="H22">
-        <v>2088</v>
+        <v>1986</v>
       </c>
       <c r="I22">
-        <v>66.9</v>
+        <v>1961</v>
       </c>
       <c r="J22">
-        <v>69.833333</v>
-      </c>
-      <c r="N22" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O22" t="str">
-        <v>proposed</v>
+        <v>1987</v>
+      </c>
+      <c r="K22">
+        <v>65.533333</v>
+      </c>
+      <c r="L22">
+        <v>66.433333</v>
       </c>
       <c r="P22" t="str">
-        <v>medium</v>
-      </c>
-      <c r="Q22">
+        <v>auto</v>
+      </c>
+      <c r="Q22" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R22" t="str">
+        <v>low</v>
+      </c>
+      <c r="S22">
         <v>1</v>
       </c>
-      <c r="R22" t="str">
+      <c r="T22" t="str">
         <v>false</v>
       </c>
     </row>
@@ -2234,7 +2694,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B23" t="str">
-        <v>e7cb6ad3-48d2-4430-a22b-6b101fc4e06b</v>
+        <v>23dce394-981c-4a8e-9eb0-aa66349c9912</v>
       </c>
       <c r="C23" t="str">
         <v>investigation</v>
@@ -2243,36 +2703,42 @@
         <v>investigation</v>
       </c>
       <c r="E23">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="F23">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="G23">
-        <v>2146</v>
+        <v>2000</v>
       </c>
       <c r="H23">
-        <v>2207</v>
+        <v>2088</v>
       </c>
       <c r="I23">
-        <v>71.766667</v>
+        <v>2001</v>
       </c>
       <c r="J23">
-        <v>73.8</v>
-      </c>
-      <c r="N23" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O23" t="str">
-        <v>proposed</v>
+        <v>2089</v>
+      </c>
+      <c r="K23">
+        <v>66.9</v>
+      </c>
+      <c r="L23">
+        <v>69.833333</v>
       </c>
       <c r="P23" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q23" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R23" t="str">
         <v>medium</v>
       </c>
-      <c r="Q23">
+      <c r="S23">
         <v>1</v>
       </c>
-      <c r="R23" t="str">
+      <c r="T23" t="str">
         <v>false</v>
       </c>
     </row>
@@ -2281,7 +2747,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B24" t="str">
-        <v>d51d2319-0725-4a70-95dc-3a3fc73871e3</v>
+        <v>e7cb6ad3-48d2-4430-a22b-6b101fc4e06b</v>
       </c>
       <c r="C24" t="str">
         <v>investigation</v>
@@ -2296,31 +2762,37 @@
         <v>15</v>
       </c>
       <c r="G24">
-        <v>2228</v>
+        <v>2146</v>
       </c>
       <c r="H24">
-        <v>2257</v>
+        <v>2207</v>
       </c>
       <c r="I24">
-        <v>74.5</v>
+        <v>2147</v>
       </c>
       <c r="J24">
-        <v>75.466667</v>
-      </c>
-      <c r="N24" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O24" t="str">
-        <v>proposed</v>
+        <v>2208</v>
+      </c>
+      <c r="K24">
+        <v>71.766667</v>
+      </c>
+      <c r="L24">
+        <v>73.8</v>
       </c>
       <c r="P24" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q24" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R24" t="str">
         <v>medium</v>
       </c>
-      <c r="Q24">
-        <v>2</v>
-      </c>
-      <c r="R24" t="str">
-        <v>true</v>
+      <c r="S24">
+        <v>1</v>
+      </c>
+      <c r="T24" t="str">
+        <v>false</v>
       </c>
     </row>
     <row r="25">
@@ -2328,7 +2800,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B25" t="str">
-        <v>f2042bd1-c034-431e-b95e-66be5387b1c1</v>
+        <v>d51d2319-0725-4a70-95dc-3a3fc73871e3</v>
       </c>
       <c r="C25" t="str">
         <v>investigation</v>
@@ -2337,37 +2809,43 @@
         <v>investigation</v>
       </c>
       <c r="E25">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F25">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G25">
-        <v>2271</v>
+        <v>2228</v>
       </c>
       <c r="H25">
-        <v>2303</v>
+        <v>2257</v>
       </c>
       <c r="I25">
-        <v>75.933333</v>
+        <v>2229</v>
       </c>
       <c r="J25">
-        <v>77</v>
-      </c>
-      <c r="N25" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O25" t="str">
-        <v>proposed</v>
+        <v>2258</v>
+      </c>
+      <c r="K25">
+        <v>74.5</v>
+      </c>
+      <c r="L25">
+        <v>75.466667</v>
       </c>
       <c r="P25" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q25" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R25" t="str">
         <v>medium</v>
       </c>
-      <c r="Q25">
-        <v>1</v>
-      </c>
-      <c r="R25" t="str">
-        <v>false</v>
+      <c r="S25">
+        <v>2</v>
+      </c>
+      <c r="T25" t="str">
+        <v>true</v>
       </c>
     </row>
     <row r="26">
@@ -2375,7 +2853,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B26" t="str">
-        <v>85ac671c-527c-4605-95e0-92479bff0b6b</v>
+        <v>f2042bd1-c034-431e-b95e-66be5387b1c1</v>
       </c>
       <c r="C26" t="str">
         <v>investigation</v>
@@ -2390,31 +2868,37 @@
         <v>16</v>
       </c>
       <c r="G26">
-        <v>2324</v>
+        <v>2271</v>
       </c>
       <c r="H26">
-        <v>2342</v>
+        <v>2303</v>
       </c>
       <c r="I26">
-        <v>77.7</v>
+        <v>2272</v>
       </c>
       <c r="J26">
-        <v>78.3</v>
-      </c>
-      <c r="N26" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O26" t="str">
-        <v>proposed</v>
+        <v>2304</v>
+      </c>
+      <c r="K26">
+        <v>75.933333</v>
+      </c>
+      <c r="L26">
+        <v>77</v>
       </c>
       <c r="P26" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q26" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R26" t="str">
         <v>medium</v>
       </c>
-      <c r="Q26">
-        <v>2</v>
-      </c>
-      <c r="R26" t="str">
-        <v>true</v>
+      <c r="S26">
+        <v>1</v>
+      </c>
+      <c r="T26" t="str">
+        <v>false</v>
       </c>
     </row>
     <row r="27">
@@ -2422,7 +2906,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B27" t="str">
-        <v>b771ee21-2ef0-4801-9c51-20c180eeba92</v>
+        <v>85ac671c-527c-4605-95e0-92479bff0b6b</v>
       </c>
       <c r="C27" t="str">
         <v>investigation</v>
@@ -2431,37 +2915,43 @@
         <v>investigation</v>
       </c>
       <c r="E27">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F27">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G27">
-        <v>2532</v>
+        <v>2324</v>
       </c>
       <c r="H27">
-        <v>2548</v>
+        <v>2342</v>
       </c>
       <c r="I27">
-        <v>84.666667</v>
+        <v>2325</v>
       </c>
       <c r="J27">
-        <v>85.2</v>
-      </c>
-      <c r="N27" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O27" t="str">
-        <v>proposed</v>
+        <v>2343</v>
+      </c>
+      <c r="K27">
+        <v>77.7</v>
+      </c>
+      <c r="L27">
+        <v>78.3</v>
       </c>
       <c r="P27" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q27" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R27" t="str">
         <v>medium</v>
       </c>
-      <c r="Q27">
-        <v>1</v>
-      </c>
-      <c r="R27" t="str">
-        <v>false</v>
+      <c r="S27">
+        <v>2</v>
+      </c>
+      <c r="T27" t="str">
+        <v>true</v>
       </c>
     </row>
     <row r="28">
@@ -2469,7 +2959,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B28" t="str">
-        <v>cc0f8c17-829e-4dd4-af32-924cd8b8d8e7</v>
+        <v>b771ee21-2ef0-4801-9c51-20c180eeba92</v>
       </c>
       <c r="C28" t="str">
         <v>investigation</v>
@@ -2478,36 +2968,42 @@
         <v>investigation</v>
       </c>
       <c r="E28">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F28">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G28">
-        <v>2589</v>
+        <v>2532</v>
       </c>
       <c r="H28">
-        <v>2612</v>
+        <v>2548</v>
       </c>
       <c r="I28">
-        <v>86.566667</v>
+        <v>2533</v>
       </c>
       <c r="J28">
-        <v>87.333333</v>
-      </c>
-      <c r="N28" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O28" t="str">
-        <v>proposed</v>
+        <v>2549</v>
+      </c>
+      <c r="K28">
+        <v>84.666667</v>
+      </c>
+      <c r="L28">
+        <v>85.2</v>
       </c>
       <c r="P28" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q28" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R28" t="str">
         <v>medium</v>
       </c>
-      <c r="Q28">
+      <c r="S28">
         <v>1</v>
       </c>
-      <c r="R28" t="str">
+      <c r="T28" t="str">
         <v>false</v>
       </c>
     </row>
@@ -2516,7 +3012,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B29" t="str">
-        <v>24a54b81-f7d9-447c-b9ba-a69009288a81</v>
+        <v>cc0f8c17-829e-4dd4-af32-924cd8b8d8e7</v>
       </c>
       <c r="C29" t="str">
         <v>investigation</v>
@@ -2525,36 +3021,42 @@
         <v>investigation</v>
       </c>
       <c r="E29">
+        <v>19</v>
+      </c>
+      <c r="F29">
+        <v>18</v>
+      </c>
+      <c r="G29">
+        <v>2589</v>
+      </c>
+      <c r="H29">
+        <v>2612</v>
+      </c>
+      <c r="I29">
+        <v>2590</v>
+      </c>
+      <c r="J29">
+        <v>2613</v>
+      </c>
+      <c r="K29">
+        <v>86.566667</v>
+      </c>
+      <c r="L29">
+        <v>87.333333</v>
+      </c>
+      <c r="P29" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q29" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R29" t="str">
+        <v>medium</v>
+      </c>
+      <c r="S29">
         <v>1</v>
       </c>
-      <c r="F29">
-        <v>0</v>
-      </c>
-      <c r="G29">
-        <v>2659</v>
-      </c>
-      <c r="H29">
-        <v>2671</v>
-      </c>
-      <c r="I29">
-        <v>88.9</v>
-      </c>
-      <c r="J29">
-        <v>89.3</v>
-      </c>
-      <c r="N29" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O29" t="str">
-        <v>proposed</v>
-      </c>
-      <c r="P29" t="str">
-        <v>high</v>
-      </c>
-      <c r="Q29">
-        <v>1</v>
-      </c>
-      <c r="R29" t="str">
+      <c r="T29" t="str">
         <v>false</v>
       </c>
     </row>
@@ -2563,7 +3065,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B30" t="str">
-        <v>f27eee5c-bf7d-42c2-b4ea-e1bb200373a4</v>
+        <v>24a54b81-f7d9-447c-b9ba-a69009288a81</v>
       </c>
       <c r="C30" t="str">
         <v>investigation</v>
@@ -2572,36 +3074,42 @@
         <v>investigation</v>
       </c>
       <c r="E30">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F30">
+        <v>0</v>
+      </c>
+      <c r="G30">
+        <v>2659</v>
+      </c>
+      <c r="H30">
+        <v>2671</v>
+      </c>
+      <c r="I30">
+        <v>2660</v>
+      </c>
+      <c r="J30">
+        <v>2672</v>
+      </c>
+      <c r="K30">
+        <v>88.9</v>
+      </c>
+      <c r="L30">
+        <v>89.3</v>
+      </c>
+      <c r="P30" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q30" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R30" t="str">
+        <v>high</v>
+      </c>
+      <c r="S30">
         <v>1</v>
       </c>
-      <c r="G30">
-        <v>2682</v>
-      </c>
-      <c r="H30">
-        <v>2707</v>
-      </c>
-      <c r="I30">
-        <v>89.666667</v>
-      </c>
-      <c r="J30">
-        <v>90.5</v>
-      </c>
-      <c r="N30" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O30" t="str">
-        <v>proposed</v>
-      </c>
-      <c r="P30" t="str">
-        <v>medium</v>
-      </c>
-      <c r="Q30">
-        <v>1</v>
-      </c>
-      <c r="R30" t="str">
+      <c r="T30" t="str">
         <v>false</v>
       </c>
     </row>
@@ -2610,7 +3118,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B31" t="str">
-        <v>2924006c-5bf1-4efa-8752-0bc683b6c667</v>
+        <v>f27eee5c-bf7d-42c2-b4ea-e1bb200373a4</v>
       </c>
       <c r="C31" t="str">
         <v>investigation</v>
@@ -2619,36 +3127,42 @@
         <v>investigation</v>
       </c>
       <c r="E31">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F31">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G31">
-        <v>2765</v>
+        <v>2682</v>
       </c>
       <c r="H31">
-        <v>2787</v>
+        <v>2707</v>
       </c>
       <c r="I31">
-        <v>92.433333</v>
+        <v>2683</v>
       </c>
       <c r="J31">
-        <v>93.166667</v>
-      </c>
-      <c r="N31" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O31" t="str">
-        <v>proposed</v>
+        <v>2708</v>
+      </c>
+      <c r="K31">
+        <v>89.666667</v>
+      </c>
+      <c r="L31">
+        <v>90.5</v>
       </c>
       <c r="P31" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q31" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R31" t="str">
         <v>medium</v>
       </c>
-      <c r="Q31">
+      <c r="S31">
         <v>1</v>
       </c>
-      <c r="R31" t="str">
+      <c r="T31" t="str">
         <v>false</v>
       </c>
     </row>
@@ -2657,7 +3171,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B32" t="str">
-        <v>c9ebde65-8056-4afc-b67b-c70c43b02bd4</v>
+        <v>2924006c-5bf1-4efa-8752-0bc683b6c667</v>
       </c>
       <c r="C32" t="str">
         <v>investigation</v>
@@ -2666,37 +3180,43 @@
         <v>investigation</v>
       </c>
       <c r="E32">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F32">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G32">
-        <v>2797</v>
+        <v>2765</v>
       </c>
       <c r="H32">
-        <v>2820</v>
+        <v>2787</v>
       </c>
       <c r="I32">
-        <v>93.5</v>
+        <v>2766</v>
       </c>
       <c r="J32">
-        <v>94.3</v>
-      </c>
-      <c r="N32" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O32" t="str">
-        <v>proposed</v>
+        <v>2788</v>
+      </c>
+      <c r="K32">
+        <v>92.433333</v>
+      </c>
+      <c r="L32">
+        <v>93.166667</v>
       </c>
       <c r="P32" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q32" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R32" t="str">
         <v>medium</v>
       </c>
-      <c r="Q32">
-        <v>2</v>
-      </c>
-      <c r="R32" t="str">
-        <v>true</v>
+      <c r="S32">
+        <v>1</v>
+      </c>
+      <c r="T32" t="str">
+        <v>false</v>
       </c>
     </row>
     <row r="33">
@@ -2704,7 +3224,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B33" t="str">
-        <v>2402180d-a771-4bd9-ab07-7dd98fcf42c4</v>
+        <v>c9ebde65-8056-4afc-b67b-c70c43b02bd4</v>
       </c>
       <c r="C33" t="str">
         <v>investigation</v>
@@ -2719,30 +3239,36 @@
         <v>4</v>
       </c>
       <c r="G33">
-        <v>2837</v>
+        <v>2797</v>
       </c>
       <c r="H33">
-        <v>2862</v>
+        <v>2820</v>
       </c>
       <c r="I33">
-        <v>94.866667</v>
+        <v>2798</v>
       </c>
       <c r="J33">
-        <v>95.7</v>
-      </c>
-      <c r="N33" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O33" t="str">
-        <v>proposed</v>
+        <v>2821</v>
+      </c>
+      <c r="K33">
+        <v>93.5</v>
+      </c>
+      <c r="L33">
+        <v>94.3</v>
       </c>
       <c r="P33" t="str">
-        <v>low</v>
-      </c>
-      <c r="Q33">
-        <v>3</v>
+        <v>auto</v>
+      </c>
+      <c r="Q33" t="str">
+        <v>proposed</v>
       </c>
       <c r="R33" t="str">
+        <v>medium</v>
+      </c>
+      <c r="S33">
+        <v>2</v>
+      </c>
+      <c r="T33" t="str">
         <v>true</v>
       </c>
     </row>
@@ -2751,7 +3277,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B34" t="str">
-        <v>dab5ef87-ae22-40c8-a077-3b82e0d921c8</v>
+        <v>2402180d-a771-4bd9-ab07-7dd98fcf42c4</v>
       </c>
       <c r="C34" t="str">
         <v>investigation</v>
@@ -2760,36 +3286,42 @@
         <v>investigation</v>
       </c>
       <c r="E34">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F34">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G34">
-        <v>2891</v>
+        <v>2837</v>
       </c>
       <c r="H34">
-        <v>3018</v>
+        <v>2862</v>
       </c>
       <c r="I34">
-        <v>96.666667</v>
+        <v>2838</v>
       </c>
       <c r="J34">
-        <v>100.9</v>
-      </c>
-      <c r="N34" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O34" t="str">
-        <v>proposed</v>
+        <v>2863</v>
+      </c>
+      <c r="K34">
+        <v>94.866667</v>
+      </c>
+      <c r="L34">
+        <v>95.7</v>
       </c>
       <c r="P34" t="str">
-        <v>medium</v>
-      </c>
-      <c r="Q34">
-        <v>4</v>
+        <v>auto</v>
+      </c>
+      <c r="Q34" t="str">
+        <v>proposed</v>
       </c>
       <c r="R34" t="str">
+        <v>low</v>
+      </c>
+      <c r="S34">
+        <v>3</v>
+      </c>
+      <c r="T34" t="str">
         <v>true</v>
       </c>
     </row>
@@ -2798,7 +3330,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B35" t="str">
-        <v>c0d7322e-9b08-4b99-ab48-59495a0af0c8</v>
+        <v>dab5ef87-ae22-40c8-a077-3b82e0d921c8</v>
       </c>
       <c r="C35" t="str">
         <v>investigation</v>
@@ -2807,36 +3339,42 @@
         <v>investigation</v>
       </c>
       <c r="E35">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F35">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G35">
-        <v>3025</v>
+        <v>2891</v>
       </c>
       <c r="H35">
-        <v>3224</v>
+        <v>3018</v>
       </c>
       <c r="I35">
-        <v>101.133333</v>
+        <v>2892</v>
       </c>
       <c r="J35">
-        <v>107.8</v>
-      </c>
-      <c r="N35" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O35" t="str">
-        <v>proposed</v>
+        <v>3019</v>
+      </c>
+      <c r="K35">
+        <v>96.666667</v>
+      </c>
+      <c r="L35">
+        <v>100.9</v>
       </c>
       <c r="P35" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q35" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R35" t="str">
         <v>medium</v>
       </c>
-      <c r="Q35">
-        <v>5</v>
-      </c>
-      <c r="R35" t="str">
+      <c r="S35">
+        <v>4</v>
+      </c>
+      <c r="T35" t="str">
         <v>true</v>
       </c>
     </row>
@@ -2845,7 +3383,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B36" t="str">
-        <v>bbd68fc5-e6f3-4dca-a65d-aced0bbebaa8</v>
+        <v>c0d7322e-9b08-4b99-ab48-59495a0af0c8</v>
       </c>
       <c r="C36" t="str">
         <v>investigation</v>
@@ -2854,36 +3392,42 @@
         <v>investigation</v>
       </c>
       <c r="E36">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F36">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G36">
-        <v>3228</v>
+        <v>3025</v>
       </c>
       <c r="H36">
-        <v>3290</v>
+        <v>3224</v>
       </c>
       <c r="I36">
-        <v>107.9</v>
+        <v>3026</v>
       </c>
       <c r="J36">
-        <v>109.966667</v>
-      </c>
-      <c r="N36" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O36" t="str">
-        <v>proposed</v>
+        <v>3225</v>
+      </c>
+      <c r="K36">
+        <v>101.133333</v>
+      </c>
+      <c r="L36">
+        <v>107.8</v>
       </c>
       <c r="P36" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q36" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R36" t="str">
         <v>medium</v>
       </c>
-      <c r="Q36">
-        <v>3</v>
-      </c>
-      <c r="R36" t="str">
+      <c r="S36">
+        <v>5</v>
+      </c>
+      <c r="T36" t="str">
         <v>true</v>
       </c>
     </row>
@@ -2892,7 +3436,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B37" t="str">
-        <v>23d6e548-ce13-4f30-a541-d1d8fe444940</v>
+        <v>bbd68fc5-e6f3-4dca-a65d-aced0bbebaa8</v>
       </c>
       <c r="C37" t="str">
         <v>investigation</v>
@@ -2901,36 +3445,42 @@
         <v>investigation</v>
       </c>
       <c r="E37">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F37">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G37">
+        <v>3228</v>
+      </c>
+      <c r="H37">
+        <v>3290</v>
+      </c>
+      <c r="I37">
+        <v>3229</v>
+      </c>
+      <c r="J37">
         <v>3291</v>
       </c>
-      <c r="H37">
-        <v>3323</v>
-      </c>
-      <c r="I37">
-        <v>110.033333</v>
-      </c>
-      <c r="J37">
-        <v>111.066732</v>
-      </c>
-      <c r="N37" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O37" t="str">
-        <v>proposed</v>
+      <c r="K37">
+        <v>107.9</v>
+      </c>
+      <c r="L37">
+        <v>109.966667</v>
       </c>
       <c r="P37" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q37" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R37" t="str">
         <v>medium</v>
       </c>
-      <c r="Q37">
+      <c r="S37">
         <v>3</v>
       </c>
-      <c r="R37" t="str">
+      <c r="T37" t="str">
         <v>true</v>
       </c>
     </row>
@@ -2939,7 +3489,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B38" t="str">
-        <v>cbc24ca0-1479-428d-a89b-b49efbb2fa82</v>
+        <v>23d6e548-ce13-4f30-a541-d1d8fe444940</v>
       </c>
       <c r="C38" t="str">
         <v>investigation</v>
@@ -2948,36 +3498,42 @@
         <v>investigation</v>
       </c>
       <c r="E38">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F38">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G38">
-        <v>3328</v>
+        <v>3291</v>
       </c>
       <c r="H38">
-        <v>3349</v>
+        <v>3323</v>
       </c>
       <c r="I38">
-        <v>111.266667</v>
+        <v>3292</v>
       </c>
       <c r="J38">
-        <v>111.966667</v>
-      </c>
-      <c r="N38" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O38" t="str">
-        <v>proposed</v>
+        <v>3324</v>
+      </c>
+      <c r="K38">
+        <v>110.033333</v>
+      </c>
+      <c r="L38">
+        <v>111.066732</v>
       </c>
       <c r="P38" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q38" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R38" t="str">
         <v>medium</v>
       </c>
-      <c r="Q38">
-        <v>4</v>
-      </c>
-      <c r="R38" t="str">
+      <c r="S38">
+        <v>3</v>
+      </c>
+      <c r="T38" t="str">
         <v>true</v>
       </c>
     </row>
@@ -2986,7 +3542,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B39" t="str">
-        <v>acfce688-6a9e-4f6e-afe5-31561dd26e13</v>
+        <v>cbc24ca0-1479-428d-a89b-b49efbb2fa82</v>
       </c>
       <c r="C39" t="str">
         <v>investigation</v>
@@ -2995,36 +3551,42 @@
         <v>investigation</v>
       </c>
       <c r="E39">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F39">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G39">
-        <v>3358</v>
+        <v>3328</v>
       </c>
       <c r="H39">
-        <v>3435</v>
+        <v>3349</v>
       </c>
       <c r="I39">
-        <v>112.266667</v>
+        <v>3329</v>
       </c>
       <c r="J39">
-        <v>114.833333</v>
-      </c>
-      <c r="N39" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O39" t="str">
-        <v>proposed</v>
+        <v>3350</v>
+      </c>
+      <c r="K39">
+        <v>111.266667</v>
+      </c>
+      <c r="L39">
+        <v>111.966667</v>
       </c>
       <c r="P39" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q39" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R39" t="str">
         <v>medium</v>
       </c>
-      <c r="Q39">
-        <v>3</v>
-      </c>
-      <c r="R39" t="str">
+      <c r="S39">
+        <v>4</v>
+      </c>
+      <c r="T39" t="str">
         <v>true</v>
       </c>
     </row>
@@ -3033,7 +3595,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B40" t="str">
-        <v>2b1a7aad-7341-43c4-a7d6-ce1814e74f42</v>
+        <v>acfce688-6a9e-4f6e-afe5-31561dd26e13</v>
       </c>
       <c r="C40" t="str">
         <v>investigation</v>
@@ -3042,36 +3604,42 @@
         <v>investigation</v>
       </c>
       <c r="E40">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F40">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G40">
-        <v>3443</v>
+        <v>3358</v>
       </c>
       <c r="H40">
-        <v>3467</v>
+        <v>3435</v>
       </c>
       <c r="I40">
-        <v>115.1</v>
+        <v>3359</v>
       </c>
       <c r="J40">
-        <v>115.9</v>
-      </c>
-      <c r="N40" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O40" t="str">
-        <v>proposed</v>
+        <v>3436</v>
+      </c>
+      <c r="K40">
+        <v>112.266667</v>
+      </c>
+      <c r="L40">
+        <v>114.833333</v>
       </c>
       <c r="P40" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q40" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R40" t="str">
         <v>medium</v>
       </c>
-      <c r="Q40">
+      <c r="S40">
         <v>3</v>
       </c>
-      <c r="R40" t="str">
+      <c r="T40" t="str">
         <v>true</v>
       </c>
     </row>
@@ -3080,7 +3648,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B41" t="str">
-        <v>0da06fa4-ebde-422b-9e75-a3acaa276729</v>
+        <v>2b1a7aad-7341-43c4-a7d6-ce1814e74f42</v>
       </c>
       <c r="C41" t="str">
         <v>investigation</v>
@@ -3089,36 +3657,42 @@
         <v>investigation</v>
       </c>
       <c r="E41">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F41">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G41">
-        <v>3475</v>
+        <v>3443</v>
       </c>
       <c r="H41">
-        <v>3504</v>
+        <v>3467</v>
       </c>
       <c r="I41">
-        <v>116.166667</v>
+        <v>3444</v>
       </c>
       <c r="J41">
-        <v>117.133333</v>
-      </c>
-      <c r="N41" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O41" t="str">
-        <v>proposed</v>
+        <v>3468</v>
+      </c>
+      <c r="K41">
+        <v>115.1</v>
+      </c>
+      <c r="L41">
+        <v>115.9</v>
       </c>
       <c r="P41" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q41" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R41" t="str">
         <v>medium</v>
       </c>
-      <c r="Q41">
-        <v>2</v>
-      </c>
-      <c r="R41" t="str">
+      <c r="S41">
+        <v>3</v>
+      </c>
+      <c r="T41" t="str">
         <v>true</v>
       </c>
     </row>
@@ -3127,7 +3701,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B42" t="str">
-        <v>12add3ee-4160-4d99-8af1-fddc8536bc9d</v>
+        <v>0da06fa4-ebde-422b-9e75-a3acaa276729</v>
       </c>
       <c r="C42" t="str">
         <v>investigation</v>
@@ -3136,36 +3710,42 @@
         <v>investigation</v>
       </c>
       <c r="E42">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F42">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G42">
-        <v>3511</v>
+        <v>3475</v>
       </c>
       <c r="H42">
-        <v>3524</v>
+        <v>3504</v>
       </c>
       <c r="I42">
-        <v>117.366667</v>
+        <v>3476</v>
       </c>
       <c r="J42">
-        <v>117.8</v>
-      </c>
-      <c r="N42" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O42" t="str">
-        <v>proposed</v>
+        <v>3505</v>
+      </c>
+      <c r="K42">
+        <v>116.166667</v>
+      </c>
+      <c r="L42">
+        <v>117.133333</v>
       </c>
       <c r="P42" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q42" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R42" t="str">
         <v>medium</v>
       </c>
-      <c r="Q42">
+      <c r="S42">
         <v>2</v>
       </c>
-      <c r="R42" t="str">
+      <c r="T42" t="str">
         <v>true</v>
       </c>
     </row>
@@ -3174,7 +3754,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B43" t="str">
-        <v>199cdbb4-2468-4a4b-a06e-e701b4417d35</v>
+        <v>12add3ee-4160-4d99-8af1-fddc8536bc9d</v>
       </c>
       <c r="C43" t="str">
         <v>investigation</v>
@@ -3183,37 +3763,43 @@
         <v>investigation</v>
       </c>
       <c r="E43">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F43">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G43">
-        <v>3569</v>
+        <v>3511</v>
       </c>
       <c r="H43">
-        <v>3646</v>
+        <v>3524</v>
       </c>
       <c r="I43">
-        <v>119.3</v>
+        <v>3512</v>
       </c>
       <c r="J43">
-        <v>121.866667</v>
-      </c>
-      <c r="N43" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O43" t="str">
-        <v>proposed</v>
+        <v>3525</v>
+      </c>
+      <c r="K43">
+        <v>117.366667</v>
+      </c>
+      <c r="L43">
+        <v>117.8</v>
       </c>
       <c r="P43" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q43" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R43" t="str">
         <v>medium</v>
       </c>
-      <c r="Q43">
-        <v>1</v>
-      </c>
-      <c r="R43" t="str">
-        <v>false</v>
+      <c r="S43">
+        <v>2</v>
+      </c>
+      <c r="T43" t="str">
+        <v>true</v>
       </c>
     </row>
     <row r="44">
@@ -3221,7 +3807,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B44" t="str">
-        <v>5042b4fa-e890-4101-9bd6-7a6e38a927ea</v>
+        <v>199cdbb4-2468-4a4b-a06e-e701b4417d35</v>
       </c>
       <c r="C44" t="str">
         <v>investigation</v>
@@ -3230,36 +3816,42 @@
         <v>investigation</v>
       </c>
       <c r="E44">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F44">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="G44">
-        <v>3727</v>
+        <v>3569</v>
       </c>
       <c r="H44">
-        <v>3770</v>
+        <v>3646</v>
       </c>
       <c r="I44">
-        <v>124.6</v>
+        <v>3570</v>
       </c>
       <c r="J44">
-        <v>126.033333</v>
-      </c>
-      <c r="N44" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O44" t="str">
-        <v>proposed</v>
+        <v>3647</v>
+      </c>
+      <c r="K44">
+        <v>119.3</v>
+      </c>
+      <c r="L44">
+        <v>121.866667</v>
       </c>
       <c r="P44" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q44" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R44" t="str">
         <v>medium</v>
       </c>
-      <c r="Q44">
+      <c r="S44">
         <v>1</v>
       </c>
-      <c r="R44" t="str">
+      <c r="T44" t="str">
         <v>false</v>
       </c>
     </row>
@@ -3268,7 +3860,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B45" t="str">
-        <v>4c934fc1-af72-4f08-b12f-8b5217fe0119</v>
+        <v>5042b4fa-e890-4101-9bd6-7a6e38a927ea</v>
       </c>
       <c r="C45" t="str">
         <v>investigation</v>
@@ -3277,37 +3869,43 @@
         <v>investigation</v>
       </c>
       <c r="E45">
+        <v>20</v>
+      </c>
+      <c r="F45">
+        <v>19</v>
+      </c>
+      <c r="G45">
+        <v>3727</v>
+      </c>
+      <c r="H45">
+        <v>3770</v>
+      </c>
+      <c r="I45">
+        <v>3728</v>
+      </c>
+      <c r="J45">
+        <v>3771</v>
+      </c>
+      <c r="K45">
+        <v>124.6</v>
+      </c>
+      <c r="L45">
+        <v>126.033333</v>
+      </c>
+      <c r="P45" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q45" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R45" t="str">
+        <v>medium</v>
+      </c>
+      <c r="S45">
         <v>1</v>
       </c>
-      <c r="F45">
-        <v>0</v>
-      </c>
-      <c r="G45">
-        <v>3775</v>
-      </c>
-      <c r="H45">
-        <v>3792</v>
-      </c>
-      <c r="I45">
-        <v>126.2</v>
-      </c>
-      <c r="J45">
-        <v>126.766667</v>
-      </c>
-      <c r="N45" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O45" t="str">
-        <v>proposed</v>
-      </c>
-      <c r="P45" t="str">
-        <v>medium</v>
-      </c>
-      <c r="Q45">
-        <v>2</v>
-      </c>
-      <c r="R45" t="str">
-        <v>true</v>
+      <c r="T45" t="str">
+        <v>false</v>
       </c>
     </row>
     <row r="46">
@@ -3315,7 +3913,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B46" t="str">
-        <v>b1541ed6-05dc-48df-b5fb-b01c49ad5c9f</v>
+        <v>4c934fc1-af72-4f08-b12f-8b5217fe0119</v>
       </c>
       <c r="C46" t="str">
         <v>investigation</v>
@@ -3324,37 +3922,43 @@
         <v>investigation</v>
       </c>
       <c r="E46">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F46">
+        <v>0</v>
+      </c>
+      <c r="G46">
+        <v>3775</v>
+      </c>
+      <c r="H46">
+        <v>3792</v>
+      </c>
+      <c r="I46">
+        <v>3776</v>
+      </c>
+      <c r="J46">
+        <v>3793</v>
+      </c>
+      <c r="K46">
+        <v>126.2</v>
+      </c>
+      <c r="L46">
+        <v>126.766667</v>
+      </c>
+      <c r="P46" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q46" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R46" t="str">
+        <v>medium</v>
+      </c>
+      <c r="S46">
         <v>2</v>
       </c>
-      <c r="G46">
-        <v>3873</v>
-      </c>
-      <c r="H46">
-        <v>3942</v>
-      </c>
-      <c r="I46">
-        <v>129.466667</v>
-      </c>
-      <c r="J46">
-        <v>131.766667</v>
-      </c>
-      <c r="N46" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O46" t="str">
-        <v>proposed</v>
-      </c>
-      <c r="P46" t="str">
-        <v>medium</v>
-      </c>
-      <c r="Q46">
-        <v>1</v>
-      </c>
-      <c r="R46" t="str">
-        <v>false</v>
+      <c r="T46" t="str">
+        <v>true</v>
       </c>
     </row>
     <row r="47">
@@ -3362,7 +3966,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B47" t="str">
-        <v>4552b990-5ec1-48ec-8e27-dc7bba72176f</v>
+        <v>b1541ed6-05dc-48df-b5fb-b01c49ad5c9f</v>
       </c>
       <c r="C47" t="str">
         <v>investigation</v>
@@ -3371,37 +3975,43 @@
         <v>investigation</v>
       </c>
       <c r="E47">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F47">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G47">
-        <v>3973</v>
+        <v>3873</v>
       </c>
       <c r="H47">
-        <v>4006</v>
+        <v>3942</v>
       </c>
       <c r="I47">
-        <v>132.8</v>
+        <v>3874</v>
       </c>
       <c r="J47">
-        <v>133.9</v>
-      </c>
-      <c r="N47" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O47" t="str">
-        <v>proposed</v>
+        <v>3943</v>
+      </c>
+      <c r="K47">
+        <v>129.466667</v>
+      </c>
+      <c r="L47">
+        <v>131.766667</v>
       </c>
       <c r="P47" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q47" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R47" t="str">
         <v>medium</v>
       </c>
-      <c r="Q47">
-        <v>4</v>
-      </c>
-      <c r="R47" t="str">
-        <v>true</v>
+      <c r="S47">
+        <v>1</v>
+      </c>
+      <c r="T47" t="str">
+        <v>false</v>
       </c>
     </row>
     <row r="48">
@@ -3409,7 +4019,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B48" t="str">
-        <v>a813a415-f192-44bb-a76f-3fa4de18a5c2</v>
+        <v>4552b990-5ec1-48ec-8e27-dc7bba72176f</v>
       </c>
       <c r="C48" t="str">
         <v>investigation</v>
@@ -3418,36 +4028,42 @@
         <v>investigation</v>
       </c>
       <c r="E48">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F48">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="G48">
-        <v>4012</v>
+        <v>3973</v>
       </c>
       <c r="H48">
-        <v>4092</v>
+        <v>4006</v>
       </c>
       <c r="I48">
-        <v>134.1</v>
+        <v>3974</v>
       </c>
       <c r="J48">
-        <v>136.766667</v>
-      </c>
-      <c r="N48" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O48" t="str">
-        <v>proposed</v>
+        <v>4007</v>
+      </c>
+      <c r="K48">
+        <v>132.8</v>
+      </c>
+      <c r="L48">
+        <v>133.9</v>
       </c>
       <c r="P48" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q48" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R48" t="str">
         <v>medium</v>
       </c>
-      <c r="Q48">
-        <v>5</v>
-      </c>
-      <c r="R48" t="str">
+      <c r="S48">
+        <v>4</v>
+      </c>
+      <c r="T48" t="str">
         <v>true</v>
       </c>
     </row>
@@ -3456,7 +4072,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B49" t="str">
-        <v>84a6cfd2-ba7a-4598-a6ea-cc3b6fc0ef70</v>
+        <v>a813a415-f192-44bb-a76f-3fa4de18a5c2</v>
       </c>
       <c r="C49" t="str">
         <v>investigation</v>
@@ -3465,36 +4081,42 @@
         <v>investigation</v>
       </c>
       <c r="E49">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F49">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G49">
-        <v>4100</v>
+        <v>4012</v>
       </c>
       <c r="H49">
-        <v>4147</v>
+        <v>4092</v>
       </c>
       <c r="I49">
-        <v>137.066667</v>
+        <v>4013</v>
       </c>
       <c r="J49">
-        <v>138.633333</v>
-      </c>
-      <c r="N49" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O49" t="str">
-        <v>proposed</v>
+        <v>4093</v>
+      </c>
+      <c r="K49">
+        <v>134.1</v>
+      </c>
+      <c r="L49">
+        <v>136.766667</v>
       </c>
       <c r="P49" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q49" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R49" t="str">
         <v>medium</v>
       </c>
-      <c r="Q49">
-        <v>6</v>
-      </c>
-      <c r="R49" t="str">
+      <c r="S49">
+        <v>5</v>
+      </c>
+      <c r="T49" t="str">
         <v>true</v>
       </c>
     </row>
@@ -3503,7 +4125,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B50" t="str">
-        <v>a6aed939-3b88-426b-9d14-526053bb54b0</v>
+        <v>84a6cfd2-ba7a-4598-a6ea-cc3b6fc0ef70</v>
       </c>
       <c r="C50" t="str">
         <v>investigation</v>
@@ -3512,36 +4134,42 @@
         <v>investigation</v>
       </c>
       <c r="E50">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F50">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="G50">
-        <v>4159</v>
+        <v>4100</v>
       </c>
       <c r="H50">
-        <v>4208</v>
+        <v>4147</v>
       </c>
       <c r="I50">
-        <v>139.033333</v>
+        <v>4101</v>
       </c>
       <c r="J50">
-        <v>140.666667</v>
-      </c>
-      <c r="N50" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O50" t="str">
-        <v>proposed</v>
+        <v>4148</v>
+      </c>
+      <c r="K50">
+        <v>137.066667</v>
+      </c>
+      <c r="L50">
+        <v>138.633333</v>
       </c>
       <c r="P50" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q50" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R50" t="str">
         <v>medium</v>
       </c>
-      <c r="Q50">
-        <v>4</v>
-      </c>
-      <c r="R50" t="str">
+      <c r="S50">
+        <v>6</v>
+      </c>
+      <c r="T50" t="str">
         <v>true</v>
       </c>
     </row>
@@ -3550,7 +4178,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B51" t="str">
-        <v>8f1bc0f4-88c3-47d3-880b-35acbd7a3916</v>
+        <v>a6aed939-3b88-426b-9d14-526053bb54b0</v>
       </c>
       <c r="C51" t="str">
         <v>investigation</v>
@@ -3559,36 +4187,42 @@
         <v>investigation</v>
       </c>
       <c r="E51">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F51">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G51">
+        <v>4159</v>
+      </c>
+      <c r="H51">
+        <v>4208</v>
+      </c>
+      <c r="I51">
+        <v>4160</v>
+      </c>
+      <c r="J51">
         <v>4209</v>
       </c>
-      <c r="H51">
-        <v>4228</v>
-      </c>
-      <c r="I51">
-        <v>140.7</v>
-      </c>
-      <c r="J51">
-        <v>141.333333</v>
-      </c>
-      <c r="N51" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O51" t="str">
-        <v>proposed</v>
+      <c r="K51">
+        <v>139.033333</v>
+      </c>
+      <c r="L51">
+        <v>140.666667</v>
       </c>
       <c r="P51" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q51" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R51" t="str">
         <v>medium</v>
       </c>
-      <c r="Q51">
+      <c r="S51">
         <v>4</v>
       </c>
-      <c r="R51" t="str">
+      <c r="T51" t="str">
         <v>true</v>
       </c>
     </row>
@@ -3597,7 +4231,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B52" t="str">
-        <v>faf421c5-f18c-4e2d-81d7-1c5857e1b6da</v>
+        <v>8f1bc0f4-88c3-47d3-880b-35acbd7a3916</v>
       </c>
       <c r="C52" t="str">
         <v>investigation</v>
@@ -3606,36 +4240,42 @@
         <v>investigation</v>
       </c>
       <c r="E52">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F52">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G52">
-        <v>4249</v>
+        <v>4209</v>
       </c>
       <c r="H52">
-        <v>4269</v>
+        <v>4228</v>
       </c>
       <c r="I52">
-        <v>142.033333</v>
+        <v>4210</v>
       </c>
       <c r="J52">
-        <v>142.7</v>
-      </c>
-      <c r="N52" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O52" t="str">
-        <v>proposed</v>
+        <v>4229</v>
+      </c>
+      <c r="K52">
+        <v>140.7</v>
+      </c>
+      <c r="L52">
+        <v>141.333333</v>
       </c>
       <c r="P52" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q52" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R52" t="str">
         <v>medium</v>
       </c>
-      <c r="Q52">
-        <v>5</v>
-      </c>
-      <c r="R52" t="str">
+      <c r="S52">
+        <v>4</v>
+      </c>
+      <c r="T52" t="str">
         <v>true</v>
       </c>
     </row>
@@ -3644,7 +4284,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B53" t="str">
-        <v>e20950a8-8d20-4f84-a78f-43729e4c613c</v>
+        <v>faf421c5-f18c-4e2d-81d7-1c5857e1b6da</v>
       </c>
       <c r="C53" t="str">
         <v>investigation</v>
@@ -3653,36 +4293,42 @@
         <v>investigation</v>
       </c>
       <c r="E53">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F53">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G53">
-        <v>4272</v>
+        <v>4249</v>
       </c>
       <c r="H53">
-        <v>4295</v>
+        <v>4269</v>
       </c>
       <c r="I53">
-        <v>142.8</v>
+        <v>4250</v>
       </c>
       <c r="J53">
-        <v>143.566667</v>
-      </c>
-      <c r="N53" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O53" t="str">
-        <v>proposed</v>
+        <v>4270</v>
+      </c>
+      <c r="K53">
+        <v>142.033333</v>
+      </c>
+      <c r="L53">
+        <v>142.7</v>
       </c>
       <c r="P53" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q53" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R53" t="str">
         <v>medium</v>
       </c>
-      <c r="Q53">
-        <v>4</v>
-      </c>
-      <c r="R53" t="str">
+      <c r="S53">
+        <v>5</v>
+      </c>
+      <c r="T53" t="str">
         <v>true</v>
       </c>
     </row>
@@ -3691,7 +4337,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B54" t="str">
-        <v>948871a8-104c-41d7-9761-524fc8a34807</v>
+        <v>e20950a8-8d20-4f84-a78f-43729e4c613c</v>
       </c>
       <c r="C54" t="str">
         <v>investigation</v>
@@ -3700,36 +4346,42 @@
         <v>investigation</v>
       </c>
       <c r="E54">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F54">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G54">
-        <v>4319</v>
+        <v>4272</v>
       </c>
       <c r="H54">
-        <v>4345</v>
+        <v>4295</v>
       </c>
       <c r="I54">
-        <v>144.366667</v>
+        <v>4273</v>
       </c>
       <c r="J54">
-        <v>145.233333</v>
-      </c>
-      <c r="N54" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O54" t="str">
-        <v>proposed</v>
+        <v>4296</v>
+      </c>
+      <c r="K54">
+        <v>142.8</v>
+      </c>
+      <c r="L54">
+        <v>143.566667</v>
       </c>
       <c r="P54" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q54" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R54" t="str">
         <v>medium</v>
       </c>
-      <c r="Q54">
+      <c r="S54">
         <v>4</v>
       </c>
-      <c r="R54" t="str">
+      <c r="T54" t="str">
         <v>true</v>
       </c>
     </row>
@@ -3738,7 +4390,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B55" t="str">
-        <v>343b9b7c-3cd7-48d7-86fd-66390f3d2ee3</v>
+        <v>948871a8-104c-41d7-9761-524fc8a34807</v>
       </c>
       <c r="C55" t="str">
         <v>investigation</v>
@@ -3747,36 +4399,42 @@
         <v>investigation</v>
       </c>
       <c r="E55">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F55">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G55">
-        <v>4409</v>
+        <v>4319</v>
       </c>
       <c r="H55">
-        <v>4430</v>
+        <v>4345</v>
       </c>
       <c r="I55">
-        <v>147.366667</v>
+        <v>4320</v>
       </c>
       <c r="J55">
-        <v>148.066667</v>
-      </c>
-      <c r="N55" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O55" t="str">
-        <v>proposed</v>
+        <v>4346</v>
+      </c>
+      <c r="K55">
+        <v>144.366667</v>
+      </c>
+      <c r="L55">
+        <v>145.233333</v>
       </c>
       <c r="P55" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q55" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R55" t="str">
         <v>medium</v>
       </c>
-      <c r="Q55">
-        <v>3</v>
-      </c>
-      <c r="R55" t="str">
+      <c r="S55">
+        <v>4</v>
+      </c>
+      <c r="T55" t="str">
         <v>true</v>
       </c>
     </row>
@@ -3785,7 +4443,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B56" t="str">
-        <v>6c55f860-bb79-4a29-8b88-f8627c805038</v>
+        <v>343b9b7c-3cd7-48d7-86fd-66390f3d2ee3</v>
       </c>
       <c r="C56" t="str">
         <v>investigation</v>
@@ -3794,36 +4452,42 @@
         <v>investigation</v>
       </c>
       <c r="E56">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F56">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G56">
-        <v>4433</v>
+        <v>4409</v>
       </c>
       <c r="H56">
-        <v>4465</v>
+        <v>4430</v>
       </c>
       <c r="I56">
-        <v>148.166667</v>
+        <v>4410</v>
       </c>
       <c r="J56">
-        <v>149.233333</v>
-      </c>
-      <c r="N56" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O56" t="str">
-        <v>proposed</v>
+        <v>4431</v>
+      </c>
+      <c r="K56">
+        <v>147.366667</v>
+      </c>
+      <c r="L56">
+        <v>148.066667</v>
       </c>
       <c r="P56" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q56" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R56" t="str">
         <v>medium</v>
       </c>
-      <c r="Q56">
+      <c r="S56">
         <v>3</v>
       </c>
-      <c r="R56" t="str">
+      <c r="T56" t="str">
         <v>true</v>
       </c>
     </row>
@@ -3832,7 +4496,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B57" t="str">
-        <v>80dd82a6-2aa5-455e-a0c3-474e80508a05</v>
+        <v>6c55f860-bb79-4a29-8b88-f8627c805038</v>
       </c>
       <c r="C57" t="str">
         <v>investigation</v>
@@ -3841,36 +4505,42 @@
         <v>investigation</v>
       </c>
       <c r="E57">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F57">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G57">
-        <v>4494</v>
+        <v>4433</v>
       </c>
       <c r="H57">
-        <v>4525</v>
+        <v>4465</v>
       </c>
       <c r="I57">
-        <v>150.233333</v>
+        <v>4434</v>
       </c>
       <c r="J57">
-        <v>151.233333</v>
-      </c>
-      <c r="N57" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O57" t="str">
-        <v>proposed</v>
+        <v>4466</v>
+      </c>
+      <c r="K57">
+        <v>148.166667</v>
+      </c>
+      <c r="L57">
+        <v>149.233333</v>
       </c>
       <c r="P57" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q57" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R57" t="str">
         <v>medium</v>
       </c>
-      <c r="Q57">
-        <v>2</v>
-      </c>
-      <c r="R57" t="str">
+      <c r="S57">
+        <v>3</v>
+      </c>
+      <c r="T57" t="str">
         <v>true</v>
       </c>
     </row>
@@ -3879,7 +4549,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B58" t="str">
-        <v>542cce36-d878-410c-807e-95347e75c189</v>
+        <v>80dd82a6-2aa5-455e-a0c3-474e80508a05</v>
       </c>
       <c r="C58" t="str">
         <v>investigation</v>
@@ -3888,36 +4558,42 @@
         <v>investigation</v>
       </c>
       <c r="E58">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F58">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G58">
-        <v>4536</v>
+        <v>4494</v>
       </c>
       <c r="H58">
-        <v>4633</v>
+        <v>4525</v>
       </c>
       <c r="I58">
-        <v>151.6</v>
+        <v>4495</v>
       </c>
       <c r="J58">
-        <v>154.866667</v>
-      </c>
-      <c r="N58" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O58" t="str">
-        <v>proposed</v>
+        <v>4526</v>
+      </c>
+      <c r="K58">
+        <v>150.233333</v>
+      </c>
+      <c r="L58">
+        <v>151.233333</v>
       </c>
       <c r="P58" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q58" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R58" t="str">
         <v>medium</v>
       </c>
-      <c r="Q58">
-        <v>3</v>
-      </c>
-      <c r="R58" t="str">
+      <c r="S58">
+        <v>2</v>
+      </c>
+      <c r="T58" t="str">
         <v>true</v>
       </c>
     </row>
@@ -3926,7 +4602,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B59" t="str">
-        <v>e96f186a-82dc-47fd-8dd4-41ede20d5b69</v>
+        <v>542cce36-d878-410c-807e-95347e75c189</v>
       </c>
       <c r="C59" t="str">
         <v>investigation</v>
@@ -3935,36 +4611,42 @@
         <v>investigation</v>
       </c>
       <c r="E59">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="F59">
+        <v>15</v>
+      </c>
+      <c r="G59">
+        <v>4536</v>
+      </c>
+      <c r="H59">
+        <v>4633</v>
+      </c>
+      <c r="I59">
+        <v>4537</v>
+      </c>
+      <c r="J59">
+        <v>4634</v>
+      </c>
+      <c r="K59">
+        <v>151.6</v>
+      </c>
+      <c r="L59">
+        <v>154.866667</v>
+      </c>
+      <c r="P59" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q59" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R59" t="str">
+        <v>medium</v>
+      </c>
+      <c r="S59">
         <v>3</v>
       </c>
-      <c r="G59">
-        <v>4993</v>
-      </c>
-      <c r="H59">
-        <v>5046</v>
-      </c>
-      <c r="I59">
-        <v>166.9</v>
-      </c>
-      <c r="J59">
-        <v>168.666667</v>
-      </c>
-      <c r="N59" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O59" t="str">
-        <v>proposed</v>
-      </c>
-      <c r="P59" t="str">
-        <v>medium</v>
-      </c>
-      <c r="Q59">
-        <v>2</v>
-      </c>
-      <c r="R59" t="str">
+      <c r="T59" t="str">
         <v>true</v>
       </c>
     </row>
@@ -3973,7 +4655,7 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B60" t="str">
-        <v>96815bbb-b8be-4b99-984e-49ad54441b0c</v>
+        <v>e96f186a-82dc-47fd-8dd4-41ede20d5b69</v>
       </c>
       <c r="C60" t="str">
         <v>investigation</v>
@@ -3982,36 +4664,42 @@
         <v>investigation</v>
       </c>
       <c r="E60">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F60">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G60">
-        <v>5048</v>
+        <v>4993</v>
       </c>
       <c r="H60">
-        <v>5538</v>
+        <v>5046</v>
       </c>
       <c r="I60">
-        <v>168.7</v>
+        <v>4994</v>
       </c>
       <c r="J60">
-        <v>185.1</v>
-      </c>
-      <c r="N60" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O60" t="str">
-        <v>proposed</v>
+        <v>5047</v>
+      </c>
+      <c r="K60">
+        <v>166.9</v>
+      </c>
+      <c r="L60">
+        <v>168.666667</v>
       </c>
       <c r="P60" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q60" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R60" t="str">
         <v>medium</v>
       </c>
-      <c r="Q60">
-        <v>5</v>
-      </c>
-      <c r="R60" t="str">
+      <c r="S60">
+        <v>2</v>
+      </c>
+      <c r="T60" t="str">
         <v>true</v>
       </c>
     </row>
@@ -4020,13 +4708,13 @@
         <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
       </c>
       <c r="B61" t="str">
-        <v>66adaa8c-e8b9-4141-83cc-15692e5e967e</v>
+        <v>96815bbb-b8be-4b99-984e-49ad54441b0c</v>
       </c>
       <c r="C61" t="str">
-        <v>escape_incomplete_censored</v>
+        <v>investigation</v>
       </c>
       <c r="D61" t="str">
-        <v>escape_incomplete_censored</v>
+        <v>investigation</v>
       </c>
       <c r="E61">
         <v>5</v>
@@ -4035,46 +4723,112 @@
         <v>4</v>
       </c>
       <c r="G61">
-        <v>5419</v>
+        <v>5048</v>
       </c>
       <c r="H61">
         <v>5538</v>
       </c>
       <c r="I61">
+        <v>5049</v>
+      </c>
+      <c r="J61">
+        <v>5539</v>
+      </c>
+      <c r="K61">
+        <v>168.7</v>
+      </c>
+      <c r="L61">
+        <v>185.1</v>
+      </c>
+      <c r="P61" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q61" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R61" t="str">
+        <v>medium</v>
+      </c>
+      <c r="S61">
+        <v>5</v>
+      </c>
+      <c r="T61" t="str">
+        <v>true</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>646e0e85-5a89-4a1d-8535-6358e211a73f</v>
+      </c>
+      <c r="B62" t="str">
+        <v>66adaa8c-e8b9-4141-83cc-15692e5e967e</v>
+      </c>
+      <c r="C62" t="str">
+        <v>escape_incomplete_censored</v>
+      </c>
+      <c r="D62" t="str">
+        <v>escape_incomplete_censored</v>
+      </c>
+      <c r="E62">
+        <v>5</v>
+      </c>
+      <c r="F62">
+        <v>4</v>
+      </c>
+      <c r="G62">
+        <v>5419</v>
+      </c>
+      <c r="H62">
+        <v>5538</v>
+      </c>
+      <c r="I62">
+        <v>5420</v>
+      </c>
+      <c r="J62">
+        <v>5539</v>
+      </c>
+      <c r="K62">
         <v>181.1</v>
       </c>
-      <c r="J61">
+      <c r="L62">
         <v>185.1</v>
       </c>
-      <c r="K61">
+      <c r="M62">
         <v>181.1</v>
       </c>
-      <c r="M61">
+      <c r="O62">
         <v>185.1</v>
       </c>
-      <c r="N61" t="str">
-        <v>auto</v>
-      </c>
-      <c r="O61" t="str">
-        <v>proposed</v>
-      </c>
-      <c r="P61" t="str">
+      <c r="P62" t="str">
+        <v>auto</v>
+      </c>
+      <c r="Q62" t="str">
+        <v>proposed</v>
+      </c>
+      <c r="R62" t="str">
         <v>medium</v>
       </c>
-      <c r="T61">
+      <c r="V62">
         <v>3</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:X62"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:V61"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:X62"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:C42"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="36.83203125" customWidth="1"/>
+    <col min="3" max="3" width="48.83203125" customWidth="1"/>
+    <col min="4" max="4" width="48.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4095,7 +4849,7 @@
         <v>exportedAt</v>
       </c>
       <c r="C2" t="str">
-        <v>2026-09-07T19:54:09.007Z</v>
+        <v>2026-09-07T20:08:18.622Z</v>
       </c>
     </row>
     <row r="3">
@@ -4536,15 +5290,22 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:C42"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:C42"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F17"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="36.83203125" customWidth="1"/>
+    <col min="3" max="3" width="48.83203125" customWidth="1"/>
+    <col min="4" max="4" width="48.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -4872,15 +5633,22 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F17"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:F17"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:U2"/>
+  <cols>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="36.83203125" customWidth="1"/>
+    <col min="3" max="3" width="48.83203125" customWidth="1"/>
+    <col min="4" max="4" width="48.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5001,6 +5769,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:U2"/>
   <ignoredErrors>
     <ignoredError numberStoredAsText="1" sqref="A1:U2"/>
   </ignoredErrors>

</xml_diff>